<commit_message>
feat: update chatbot backend and frontend with latest changes
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/MeDay_Treatments_Data_finalalmost.xlsx
+++ b/backend/MeDay_Treatments_Data_finalalmost.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Treatments" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recommendation_Questions" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recommendation_Scoring" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FAQ" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forward_Topics" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes_Discrepancies" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Categories" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Treatments" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Recommendation_Questions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Recommendation_Scoring" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="FAQ" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Forward_Topics" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Notes_Discrepancies" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1177,7 +1177,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L136"/>
+  <dimension ref="A1:S136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1255,6 +1255,41 @@
           <t>source</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>preparation</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>aftercare</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>downtime</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>pain_level</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>sessions_recommended</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>results_longevity</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>what_to_expect</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -1297,6 +1332,41 @@
           <t>אתר</t>
         </is>
       </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>אין הכנה מיוחדת; מומלץ להגיע ללא ציפוי קודם אם מעוניינים בהסרה עצמאית מראש.</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>מומלץ להזין את העור בקרם ידיים/רגליים ולהימנע מחשיפה ממושכת למים חמים מיד לאחר הטיפול.</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>אין זמן החלמה — ניתן לחזור לשגרה מיד.</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>טיפול נעים ולא כואב.</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>מומלץ ריענון כל 2-3 שבועות לשמירה על מראה מטופח.</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>לק רגיל מחזיק מספר ימים; לק ג'ל נשמר בדרך כלל כשבועיים-שלושה.</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>מניקור הכולל מניקור ידני ומכשירי והסרת ציפוי ישן.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -1339,6 +1409,41 @@
           <t>אתר</t>
         </is>
       </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>אין הכנה מיוחדת; מומלץ להגיע ללא ציפוי קודם אם מעוניינים בהסרה עצמאית מראש.</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>מומלץ להזין את העור בקרם ידיים/רגליים ולהימנע מחשיפה ממושכת למים חמים מיד לאחר הטיפול.</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>אין זמן החלמה — ניתן לחזור לשגרה מיד.</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>טיפול נעים ולא כואב.</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>מומלץ ריענון כל 2-3 שבועות לשמירה על מראה מטופח.</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>לק ג'ל נשמר בדרך כלל כשבועיים-שלושה.</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>לק ג'ל הכולל הסרת ציפוי ישן, מניקור, תיקון מבנה וציפוי בג'ל.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -1381,6 +1486,41 @@
           <t>אתר</t>
         </is>
       </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>אין הכנה מיוחדת; מומלץ להגיע ללא ציפוי קודם אם מעוניינים בהסרה עצמאית מראש.</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>מומלץ להזין את העור בקרם ידיים/רגליים ולהימנע מחשיפה ממושכת למים חמים מיד לאחר הטיפול.</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>אין זמן החלמה — ניתן לחזור לשגרה מיד.</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>טיפול נעים ולא כואב.</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>מומלץ ריענון כל 2-3 שבועות לשמירה על מראה מטופח.</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>לק רגיל מחזיק מספר ימים; לק ג'ל נשמר בדרך כלל כשבועיים-שלושה.</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>עיצוב ופיסול ציפורן הכולל בנייה, עיצוב וציפוי בג'ל.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -1425,6 +1565,41 @@
           <t>שניהם</t>
         </is>
       </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>אין הכנה מיוחדת; מומלץ להגיע ללא ציפוי קודם אם מעוניינים בהסרה עצמאית מראש.</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>מומלץ להזין את העור בקרם ידיים/רגליים ולהימנע מחשיפה ממושכת למים חמים מיד לאחר הטיפול.</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>אין זמן החלמה — ניתן לחזור לשגרה מיד.</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>טיפול נעים ולא כואב.</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>מומלץ ריענון כל 2-3 שבועות לשמירה על מראה מטופח.</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>לק רגיל מחזיק מספר ימים; לק ג'ל נשמר בדרך כלל כשבועיים-שלושה.</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>פדיקור אסתטי עם מריחת לק — ניקוי, הסרת עור יבש ועיצוב הציפורניים.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -1469,6 +1644,41 @@
           <t>שניהם</t>
         </is>
       </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>אין הכנה מיוחדת; מומלץ להגיע ללא ציפוי קודם אם מעוניינים בהסרה עצמאית מראש.</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>מומלץ להזין את העור בקרם ידיים/רגליים ולהימנע מחשיפה ממושכת למים חמים מיד לאחר הטיפול.</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>אין זמן החלמה — ניתן לחזור לשגרה מיד.</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>טיפול נעים ולא כואב.</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>מומלץ ריענון כל 2-3 שבועות לשמירה על מראה מטופח.</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>לק ג'ל נשמר בדרך כלל כשבועיים-שלושה.</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>פדיקור אסתטי עם לק ג'ל — ניקוי, הסרת עור יבש ועיצוב הציפורניים.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -1515,6 +1725,41 @@
       <c r="L7" s="3" t="inlineStr">
         <is>
           <t>שניהם</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>אין הכנה מיוחדת; מומלץ להגיע ללא ציפוי קודם אם מעוניינים בהסרה עצמאית מראש.</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>מומלץ להזין את העור בקרם ידיים/רגליים ולהימנע מחשיפה ממושכת למים חמים מיד לאחר הטיפול.</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>אין זמן החלמה — ניתן לחזור לשגרה מיד.</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>טיפול נעים ולא כואב.</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>מומלץ ריענון כל 2-3 שבועות לשמירה על מראה מטופח.</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>לק רגיל מחזיק מספר ימים; לק ג'ל נשמר בדרך כלל כשבועיים-שלושה.</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>פדיקור טיפולי עם לק/לק ג'ל, כולל טיפול בכף הרגל.</t>
         </is>
       </c>
     </row>
@@ -2917,6 +3162,41 @@
           <t>אתר</t>
         </is>
       </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>מומלץ להגיע ללא איפור ולהימנע מחומצות, רטינול או פילינג ביתי מספר ימים לפני הטיפול. לפני טיפולים מבוססי אור/לייזר יש להימנע מחשיפה ממושכת לשמש ומשיזוף.</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>מומלץ להימנע מאיפור למשך מספר שעות, להקפיד על קרם הגנה SPF, ולהימנע מחשיפה ישירה לשמש, סאונה ומאמץ מזיע ביום-יומיים הראשונים.</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>אין זמן החלמה משמעותי — ניתן לחזור לשגרה מיד.</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>לרוב נעים; ייתכן אי-נוחות קלה בשלב ניקוז הקומדונים.</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>ניתן כטיפול בודד; לתוצאה מיטבית מומלצת תחזוקה תקופתית.</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>תחושת רעננות מיידית; לתוצאה מתמשכת מומלצת תחזוקה קבועה.</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>ניקוי פנים קלאסי הכולל פילינג, ניקוז קומדונים, טיהור וחיטוי ואיזון לחות; מתאים לכל גיל וסוג עור.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
@@ -2967,6 +3247,41 @@
           <t>אתר</t>
         </is>
       </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>מומלץ להגיע ללא איפור ולהימנע מחומצות, רטינול או פילינג ביתי מספר ימים לפני הטיפול. לפני טיפולים מבוססי אור/לייזר יש להימנע מחשיפה ממושכת לשמש ומשיזוף.</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>מומלץ להימנע מאיפור למשך מספר שעות, להקפיד על קרם הגנה SPF, ולהימנע מחשיפה ישירה לשמש, סאונה ומאמץ מזיע ביום-יומיים הראשונים.</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>אין זמן החלמה משמעותי — ניתן לחזור לשגרה מיד.</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>לרוב נעים; ייתכן אי-נוחות קלה בשלב ניקוז הקומדונים.</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>ניתן כטיפול בודד; לתוצאה מיטבית מומלצת תחזוקה תקופתית.</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>תחושת רעננות מיידית; לתוצאה מתמשכת מומלצת תחזוקה קבועה.</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>טיפול פנים מותאם לעור הגברי — ניקוי עמוק, איזון שומניות והרגעה, כולל הסרת שיער בשעווה מהאף והאוזניים.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
@@ -3017,6 +3332,41 @@
           <t>אתר</t>
         </is>
       </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>מומלץ להגיע ללא איפור ולהימנע מחומצות, רטינול או פילינג ביתי מספר ימים לפני הטיפול. לפני טיפולים מבוססי אור/לייזר יש להימנע מחשיפה ממושכת לשמש ומשיזוף.</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>מומלץ להימנע מאיפור למשך מספר שעות, להקפיד על קרם הגנה SPF, ולהימנע מחשיפה ישירה לשמש, סאונה ומאמץ מזיע ביום-יומיים הראשונים.</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>אין זמן החלמה.</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>נעים ולא כואב.</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>ניתן כטיפול בודד; לתוצאה מיטבית מומלצת תחזוקה תקופתית.</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>תחושת רעננות מיידית; לתוצאה מתמשכת מומלצת תחזוקה קבועה.</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>עיסוי פנים קוסמטי מפנק להרמה, מיצוק ושיפור קווי המתאר של הפנים.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
@@ -3067,6 +3417,41 @@
           <t>אתר</t>
         </is>
       </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>מומלץ להגיע ללא איפור ולהימנע מחומצות, רטינול או פילינג ביתי מספר ימים לפני הטיפול. לפני טיפולים מבוססי אור/לייזר יש להימנע מחשיפה ממושכת לשמש ומשיזוף.</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>מומלץ להימנע מאיפור למשך מספר שעות, להקפיד על קרם הגנה SPF, ולהימנע מחשיפה ישירה לשמש, סאונה ומאמץ מזיע ביום-יומיים הראשונים.</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>אין זמן החלמה — מתאים ממש לפני אירוע.</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>נעים ולא כואב.</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>מתאים כטיפול בודד לקראת אירוע.</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>תחושת רעננות מיידית; לתוצאה מתמשכת מומלצת תחזוקה קבועה.</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>טיפול זוהר לפני אירוע: ניקוי, החדרת לחות ועיסוי מעצב בשילוב אולטרסאונד ופילינג יהלום.</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
@@ -3119,6 +3504,41 @@
       <c r="L46" s="3" t="inlineStr">
         <is>
           <t>אתר</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>מומלץ להגיע ללא איפור ולהימנע מחומצות, רטינול או פילינג ביתי מספר ימים לפני הטיפול. לפני טיפולים מבוססי אור/לייזר יש להימנע מחשיפה ממושכת לשמש ומשיזוף.</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>מומלץ להימנע מאיפור למשך מספר שעות, להקפיד על קרם הגנה SPF, ולהימנע מחשיפה ישירה לשמש, סאונה ומאמץ מזיע ביום-יומיים הראשונים.</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>ייתכן אודם קל שחולף תוך שעות עד יום-יומיים.</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>אי-נוחות קלה; ניתן להשתמש בחומר הרדמה מקומי.</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>מומלצת סדרת טיפולים לתוצאה מיטבית, בהתאם לייעוץ.</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>תחושת רעננות מיידית; לתוצאה מתמשכת מומלצת תחזוקה קבועה.</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>מזותרפיה קוסמטית עם מחטים זעירות להחדרת חומרים פעילים למיצוק, הבהרה וחידוש מרקם העור.</t>
         </is>
       </c>
     </row>
@@ -3171,6 +3591,41 @@
           <t>אתר</t>
         </is>
       </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>מומלץ להגיע ללא איפור ולהימנע מחומצות, רטינול או פילינג ביתי מספר ימים לפני הטיפול. לפני טיפולים מבוססי אור/לייזר יש להימנע מחשיפה ממושכת לשמש ומשיזוף.</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>מומלץ להימנע מאיפור למשך מספר שעות, להקפיד על קרם הגנה SPF, ולהימנע מחשיפה ישירה לשמש, סאונה ומאמץ מזיע ביום-יומיים הראשונים.</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>אין זמן החלמה משמעותי; ייתכן אודם קל וחולף.</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>תחושת חום נעימה במהלך הטיפול.</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>ניתן כטיפול בודד; לתוצאה מיטבית מומלצת תחזוקה תקופתית.</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>תחושת רעננות מיידית; לתוצאה מתמשכת מומלצת תחזוקה קבועה.</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>טיפול גלי רדיו (RF) למיצוק ושיפור מרקם; מעודד יצירת קולגן בשכבות העמוקות.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
@@ -3225,6 +3680,41 @@
           <t>אתר</t>
         </is>
       </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>מומלץ להגיע ללא איפור ולהימנע מחומצות, רטינול או פילינג ביתי מספר ימים לפני הטיפול. לפני טיפולים מבוססי אור/לייזר יש להימנע מחשיפה ממושכת לשמש ומשיזוף.</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>מומלץ להימנע מאיפור למשך מספר שעות, להקפיד על קרם הגנה SPF, ולהימנע מחשיפה ישירה לשמש, סאונה ומאמץ מזיע ביום-יומיים הראשונים.</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>ייתכן אודם קל שחולף תוך שעות עד יום-יומיים.</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>תחושת חום ועקצוץ קלה וחולפת.</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>מומלצת סדרת טיפולים לתוצאה מיטבית, בהתאם לייעוץ.</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>תחושת רעננות מיידית; לתוצאה מתמשכת מומלצת תחזוקה קבועה.</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>טיפול IPL לחידוש העור למראה אחיד ומוצק; מתקן גוון לא אחיד ונקבוביות.</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
@@ -3277,6 +3767,41 @@
       <c r="L49" s="3" t="inlineStr">
         <is>
           <t>אתר</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>מומלץ להגיע ללא איפור ולהימנע מחומצות, רטינול או פילינג ביתי מספר ימים לפני הטיפול. לפני טיפולים מבוססי אור/לייזר יש להימנע מחשיפה ממושכת לשמש ומשיזוף.</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>מומלץ להימנע מאיפור למשך מספר שעות, להקפיד על קרם הגנה SPF, ולהימנע מחשיפה ישירה לשמש, סאונה ומאמץ מזיע ביום-יומיים הראשונים.</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>ייתכן אודם קל שחולף תוך שעות עד יום-יומיים.</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>תחושת חום ועקצוץ קלה וחולפת.</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>מומלצת סדרת טיפולים לטיפול באקנה, בהתאם לייעוץ.</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>תחושת רעננות מיידית; לתוצאה מתמשכת מומלצת תחזוקה קבועה.</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>טיפול IPL להעלמת אקנה והפחתת דלקתיות; מתאים לאקנה בדרגות 1-2.</t>
         </is>
       </c>
     </row>
@@ -3329,6 +3854,41 @@
           <t>אתר</t>
         </is>
       </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>מומלץ להגיע ללא איפור ולהימנע מחומצות, רטינול או פילינג ביתי מספר ימים לפני הטיפול. לפני טיפולים מבוססי אור/לייזר יש להימנע מחשיפה ממושכת לשמש ומשיזוף.</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>מומלץ להימנע מאיפור למשך מספר שעות, להקפיד על קרם הגנה SPF, ולהימנע מחשיפה ישירה לשמש, סאונה ומאמץ מזיע ביום-יומיים הראשונים.</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>ייתכן אודם קל שחולף במהירות.</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>עקצוץ וחום קלים.</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>ניתן כטיפול בודד; לתוצאה מיטבית מומלצת תחזוקה תקופתית.</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>תחושת רעננות מיידית; לתוצאה מתמשכת מומלצת תחזוקה קבועה.</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>ניקוי יסודי בשילוב פילינג יהלום עדין לשיפור מרקם, הבהרה ומראה זוהר.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
@@ -3381,6 +3941,41 @@
       <c r="L51" s="3" t="inlineStr">
         <is>
           <t>אתר</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>מומלץ להגיע ללא איפור ולהימנע מחומצות, רטינול או פילינג ביתי מספר ימים לפני הטיפול. לפני טיפולים מבוססי אור/לייזר יש להימנע מחשיפה ממושכת לשמש ומשיזוף.</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>מומלץ להימנע מאיפור למשך מספר שעות, להקפיד על קרם הגנה SPF, ולהימנע מחשיפה ישירה לשמש, סאונה ומאמץ מזיע ביום-יומיים הראשונים.</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>ייתכן אודם וקילוף קל למספר ימים בהתאם לעומק הפילינג.</t>
+        </is>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>עקצוץ וחום קלים; ייתכן קילוף עדין בימים שאחרי.</t>
+        </is>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>מבוצע כסדרה מותאמת אישית לפי ייעוץ.</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>תחושת רעננות מיידית; לתוצאה מתמשכת מומלצת תחזוקה קבועה.</t>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>סדרת פילינגים כימיים מתקדמים ומותאמים אישית לאקנה, פיגמנטציה והזדקנות.</t>
         </is>
       </c>
     </row>
@@ -3435,6 +4030,41 @@
       <c r="L52" s="3" t="inlineStr">
         <is>
           <t>אתר</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>מומלץ להגיע ללא איפור ולהימנע מחומצות, רטינול או פילינג ביתי מספר ימים לפני הטיפול. לפני טיפולים מבוססי אור/לייזר יש להימנע מחשיפה ממושכת לשמש ומשיזוף.</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>מומלץ להימנע מאיפור למשך מספר שעות, להקפיד על קרם הגנה SPF, ולהימנע מחשיפה ישירה לשמש, סאונה ומאמץ מזיע ביום-יומיים הראשונים.</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>ייתכן אודם קל שחולף תוך שעות עד יום-יומיים.</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>עקצוץ וחום קלים.</t>
+        </is>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>מומלצת סדרת טיפולים לתוצאה מיטבית, בהתאם לייעוץ.</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>תחושת רעננות מיידית; לתוצאה מתמשכת מומלצת תחזוקה קבועה.</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>טיפול הצערה עוצמתי עם תכשירים קוסמטיים מתקדמים למתיחה, מילוי וחידוש העור.</t>
         </is>
       </c>
     </row>
@@ -3487,6 +4117,41 @@
           <t>מחירון בלבד - לא מופיע באתר הנוכחי, יתכן וזהה ל'מידיי קלאסי'</t>
         </is>
       </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>מומלץ להגיע ללא איפור ולהימנע מחומצות, רטינול או פילינג ביתי מספר ימים לפני הטיפול. לפני טיפולים מבוססי אור/לייזר יש להימנע מחשיפה ממושכת לשמש ומשיזוף.</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>מומלץ להימנע מאיפור למשך מספר שעות, להקפיד על קרם הגנה SPF, ולהימנע מחשיפה ישירה לשמש, סאונה ומאמץ מזיע ביום-יומיים הראשונים.</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>אין זמן החלמה משמעותי — ניתן לחזור לשגרה מיד.</t>
+        </is>
+      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>לרוב נעים; ייתכן אי-נוחות קלה בשלב ניקוז הקומדונים.</t>
+        </is>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>ניתן כטיפול בודד; לתוצאה מיטבית מומלצת תחזוקה תקופתית.</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>תחושת רעננות מיידית; לתוצאה מתמשכת מומלצת תחזוקה קבועה.</t>
+        </is>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>ניקוי עמוק מותאם אישית לפי סוג העור לשיפור מרקם ומראה רענן.</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
@@ -3537,6 +4202,41 @@
           <t>מחירון בלבד - לא מופיע באתר הנוכחי</t>
         </is>
       </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>מומלץ להגיע ללא איפור ולהימנע מחומצות, רטינול או פילינג ביתי מספר ימים לפני הטיפול. לפני טיפולים מבוססי אור/לייזר יש להימנע מחשיפה ממושכת לשמש ומשיזוף.</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>מומלץ להימנע מאיפור למשך מספר שעות, להקפיד על קרם הגנה SPF, ולהימנע מחשיפה ישירה לשמש, סאונה ומאמץ מזיע ביום-יומיים הראשונים.</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>אין זמן החלמה.</t>
+        </is>
+      </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>נעים ולא כואב — ללא הזרקות.</t>
+        </is>
+      </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>ניתן כטיפול בודד; לתוצאה מיטבית מומלצת תחזוקה תקופתית.</t>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>תחושת רעננות מיידית; לתוצאה מתמשכת מומלצת תחזוקה קבועה.</t>
+        </is>
+      </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>החדרת חומרים פעילים לעומק העור באלקטרופורציה (ללא הזרקות) לזוהר, לחות ורעננות.</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
@@ -3587,6 +4287,41 @@
           <t>אתר</t>
         </is>
       </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>מומלץ להגיע רגוע, להימנע מארוחה כבדה כשעה לפני הטיפול, ולעדכן את המטפל/ת על אזורים רגישים או כאב.</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>מומלץ לשתות הרבה מים לאחר העיסוי, לנוח ולהימנע ממאמץ גופני אינטנסיבי באותו יום.</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>אין זמן החלמה — ניתן לחזור לשגרה מיד.</t>
+        </is>
+      </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>לחץ בינוני ומרגיע; ניתן להתאים את העוצמה מול המטפל/ת.</t>
+        </is>
+      </c>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>ניתן כטיפול בודד או כסדרה לתחזוקה לפי הצורך.</t>
+        </is>
+      </c>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>תחושת ההרפיה מורגשת מיד; לתחזוקה מתמשכת מומלץ עיסוי קבוע.</t>
+        </is>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>עיסוי שוודי עדין עם שמנים להרגעה, שחרור מתחים ושיפור זרימת הדם.</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
@@ -3633,6 +4368,41 @@
       <c r="L56" s="3" t="inlineStr">
         <is>
           <t>שניהם - מלא בלבד</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>מומלץ להגיע רגוע, להימנע מארוחה כבדה כשעה לפני הטיפול, ולעדכן את המטפל/ת על אזורים רגישים או כאב.</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>מומלץ לשתות הרבה מים לאחר העיסוי, לנוח ולהימנע ממאמץ גופני אינטנסיבי באותו יום.</t>
+        </is>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>אין זמן החלמה — ניתן לחזור לשגרה מיד.</t>
+        </is>
+      </c>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t>עדין ונעים עם חום מרגיע.</t>
+        </is>
+      </c>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>ניתן כטיפול בודד או כסדרה לתחזוקה לפי הצורך.</t>
+        </is>
+      </c>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>תחושת ההרפיה מורגשת מיד; לתחזוקה מתמשכת מומלץ עיסוי קבוע.</t>
+        </is>
+      </c>
+      <c r="S56" t="inlineStr">
+        <is>
+          <t>עיסוי באבנים חמות המשלב חום מרגיע לשחרור שרירים תפוסים והפגת מתחים.</t>
         </is>
       </c>
     </row>
@@ -3681,6 +4451,41 @@
           <t>אתר</t>
         </is>
       </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>מומלץ להגיע רגוע, להימנע מארוחה כבדה כשעה לפני הטיפול, ולעדכן את המטפל/ת על אזורים רגישים או כאב.</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>מומלץ לשתות הרבה מים לאחר העיסוי, לנוח ולהימנע ממאמץ גופני אינטנסיבי באותו יום.</t>
+        </is>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>אין זמן החלמה — ניתן לחזור לשגרה מיד.</t>
+        </is>
+      </c>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t>לחץ חזק יותר על נקודות בגוף; ייתכן אי-נוחות קלה.</t>
+        </is>
+      </c>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>ניתן כטיפול בודד או כסדרה לתחזוקה לפי הצורך.</t>
+        </is>
+      </c>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t>תחושת ההרפיה מורגשת מיד; לתחזוקה מתמשכת מומלץ עיסוי קבוע.</t>
+        </is>
+      </c>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t>עיסוי תאילנדי בלחץ על נקודות בגוף לשיפור זרימת אנרגיה, גמישות והפחתת מתח.</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
@@ -3727,6 +4532,41 @@
           <t>אתר</t>
         </is>
       </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>מומלץ להגיע רגוע, להימנע מארוחה כבדה כשעה לפני הטיפול, ולעדכן את המטפל/ת על אזורים רגישים או כאב.</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>מומלץ לשתות הרבה מים לאחר העיסוי, לנוח ולהימנע ממאמץ גופני אינטנסיבי באותו יום.</t>
+        </is>
+      </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>אין זמן החלמה — ניתן לחזור לשגרה מיד.</t>
+        </is>
+      </c>
+      <c r="P58" t="inlineStr">
+        <is>
+          <t>לחץ בינוני ומרגיע; ניתן להתאים את העוצמה מול המטפל/ת.</t>
+        </is>
+      </c>
+      <c r="Q58" t="inlineStr">
+        <is>
+          <t>ניתן כטיפול בודד או כסדרה לתחזוקה לפי הצורך.</t>
+        </is>
+      </c>
+      <c r="R58" t="inlineStr">
+        <is>
+          <t>תחושת ההרפיה מורגשת מיד; לתחזוקה מתמשכת מומלץ עיסוי קבוע.</t>
+        </is>
+      </c>
+      <c r="S58" t="inlineStr">
+        <is>
+          <t>שיאצו יפני בלחיצות ממוקדות על נקודות אנרגיה לאיזון ושיפור זרימת הדם.</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
@@ -3777,6 +4617,41 @@
           <t>שניהם</t>
         </is>
       </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>מומלץ להגיע רגוע, להימנע מארוחה כבדה כשעה לפני הטיפול, ולעדכן את המטפל/ת על אזורים רגישים או כאב.</t>
+        </is>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>מומלץ לשתות הרבה מים לאחר העיסוי, לנוח ולהימנע ממאמץ גופני אינטנסיבי באותו יום.</t>
+        </is>
+      </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>אין זמן החלמה — ניתן לחזור לשגרה מיד.</t>
+        </is>
+      </c>
+      <c r="P59" t="inlineStr">
+        <is>
+          <t>עיסוי אינטנסיבי בלחץ חזק; ייתכן אי-נוחות באזורים תפוסים. מומלץ לתאם עוצמה עם המטפל/ת.</t>
+        </is>
+      </c>
+      <c r="Q59" t="inlineStr">
+        <is>
+          <t>ניתן כטיפול בודד או כסדרה לתחזוקה לפי הצורך.</t>
+        </is>
+      </c>
+      <c r="R59" t="inlineStr">
+        <is>
+          <t>תחושת ההרפיה מורגשת מיד; לתחזוקה מתמשכת מומלץ עיסוי קבוע.</t>
+        </is>
+      </c>
+      <c r="S59" t="inlineStr">
+        <is>
+          <t>עיסוי רקמות עמוק לשחרור מתחים כרוניים ואזורים כואבים.</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
@@ -3823,6 +4698,41 @@
       <c r="L60" s="3" t="inlineStr">
         <is>
           <t>שניהם</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>מומלץ להגיע רגוע, להימנע מארוחה כבדה כשעה לפני הטיפול, ולעדכן את המטפל/ת על אזורים רגישים או כאב.</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>מומלץ לשתות הרבה מים לאחר העיסוי, לנוח ולהימנע ממאמץ גופני אינטנסיבי באותו יום.</t>
+        </is>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>אין זמן החלמה — ניתן לחזור לשגרה מיד.</t>
+        </is>
+      </c>
+      <c r="P60" t="inlineStr">
+        <is>
+          <t>לחץ בינוני ומרגיע; ניתן להתאים את העוצמה מול המטפל/ת.</t>
+        </is>
+      </c>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>ניתן כטיפול בודד או כסדרה לתחזוקה לפי הצורך.</t>
+        </is>
+      </c>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>תחושת ההרפיה מורגשת מיד; לתחזוקה מתמשכת מומלץ עיסוי קבוע.</t>
+        </is>
+      </c>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t>עיסוי קצוות — ראש, צוואר, ידיים וכפות רגליים — מרגיע ומפנק.</t>
         </is>
       </c>
     </row>
@@ -3871,6 +4781,41 @@
           <t>אתר</t>
         </is>
       </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>מומלץ להגיע רגוע, להימנע מארוחה כבדה כשעה לפני הטיפול, ולעדכן את המטפל/ת על אזורים רגישים או כאב.</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>מומלץ לשתות הרבה מים לאחר העיסוי, לנוח ולהימנע ממאמץ גופני אינטנסיבי באותו יום.</t>
+        </is>
+      </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>אין זמן החלמה — ניתן לחזור לשגרה מיד.</t>
+        </is>
+      </c>
+      <c r="P61" t="inlineStr">
+        <is>
+          <t>לחץ ממוקד וחזק יותר על אזורים תפוסים.</t>
+        </is>
+      </c>
+      <c r="Q61" t="inlineStr">
+        <is>
+          <t>ניתן כטיפול בודד או כסדרה לתחזוקה לפי הצורך.</t>
+        </is>
+      </c>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>תחושת ההרפיה מורגשת מיד; לתחזוקה מתמשכת מומלץ עיסוי קבוע.</t>
+        </is>
+      </c>
+      <c r="S61" t="inlineStr">
+        <is>
+          <t>עיסוי ממוקד לכתפיים, גב וצוואר להקלה על מתח וכאב מאורח חיים יושבני.</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
@@ -3917,6 +4862,41 @@
       <c r="L62" s="3" t="inlineStr">
         <is>
           <t>שניהם</t>
+        </is>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>מומלץ להגיע רגוע, להימנע מארוחה כבדה כשעה לפני הטיפול, ולעדכן את המטפל/ת על אזורים רגישים או כאב.</t>
+        </is>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>מומלץ לשתות הרבה מים לאחר העיסוי, לנוח ולהימנע ממאמץ גופני אינטנסיבי באותו יום.</t>
+        </is>
+      </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>אין זמן החלמה — ניתן לחזור לשגרה מיד.</t>
+        </is>
+      </c>
+      <c r="P62" t="inlineStr">
+        <is>
+          <t>לחץ בינוני ומרגיע; ניתן להתאים את העוצמה מול המטפל/ת.</t>
+        </is>
+      </c>
+      <c r="Q62" t="inlineStr">
+        <is>
+          <t>ניתן כטיפול בודד או כסדרה לתחזוקה לפי הצורך.</t>
+        </is>
+      </c>
+      <c r="R62" t="inlineStr">
+        <is>
+          <t>תחושת ההרפיה מורגשת מיד; לתחזוקה מתמשכת מומלץ עיסוי קבוע.</t>
+        </is>
+      </c>
+      <c r="S62" t="inlineStr">
+        <is>
+          <t>עיסוי פנים וקרקפת מרגיע לשחרור מתחים ולהפחתת סימני עייפות.</t>
         </is>
       </c>
     </row>
@@ -3965,6 +4945,41 @@
           <t>שניהם</t>
         </is>
       </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>מומלץ להגיע רגוע, להימנע מארוחה כבדה כשעה לפני הטיפול, ולעדכן את המטפל/ת על אזורים רגישים או כאב.</t>
+        </is>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>מומלץ לשתות הרבה מים לאחר העיסוי, לנוח ולהימנע ממאמץ גופני אינטנסיבי באותו יום.</t>
+        </is>
+      </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>אין זמן החלמה — ניתן לחזור לשגרה מיד.</t>
+        </is>
+      </c>
+      <c r="P63" t="inlineStr">
+        <is>
+          <t>לחץ בינוני ומרגיע; ניתן להתאים את העוצמה מול המטפל/ת.</t>
+        </is>
+      </c>
+      <c r="Q63" t="inlineStr">
+        <is>
+          <t>ניתן כטיפול בודד או כסדרה לתחזוקה לפי הצורך.</t>
+        </is>
+      </c>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>תחושת ההרפיה מורגשת מיד; לתחזוקה מתמשכת מומלץ עיסוי קבוע.</t>
+        </is>
+      </c>
+      <c r="S63" t="inlineStr">
+        <is>
+          <t>עיסוי כפות רגליים מרגיע ומפנק לשחרור מתחים.</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
@@ -4015,6 +5030,41 @@
           <t>אתר</t>
         </is>
       </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>מומלץ להגיע רגוע, להימנע מארוחה כבדה כשעה לפני הטיפול, ולעדכן את המטפל/ת על אזורים רגישים או כאב.</t>
+        </is>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>מומלץ לשתות הרבה מים לאחר העיסוי, לנוח ולהימנע ממאמץ גופני אינטנסיבי באותו יום.</t>
+        </is>
+      </c>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t>אין זמן החלמה — ניתן לחזור לשגרה מיד.</t>
+        </is>
+      </c>
+      <c r="P64" t="inlineStr">
+        <is>
+          <t>עיסוי ממוקד בעוצמה בינונית-חזקה.</t>
+        </is>
+      </c>
+      <c r="Q64" t="inlineStr">
+        <is>
+          <t>ניתן כטיפול בודד או כסדרה לתחזוקה לפי הצורך.</t>
+        </is>
+      </c>
+      <c r="R64" t="inlineStr">
+        <is>
+          <t>תחושת ההרפיה מורגשת מיד; לתחזוקה מתמשכת מומלץ עיסוי קבוע.</t>
+        </is>
+      </c>
+      <c r="S64" t="inlineStr">
+        <is>
+          <t>עיסוי ספורטאים לשיקום שרירים, מניעת פציעות ושיפור ביצועים.</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
@@ -4065,6 +5115,41 @@
       <c r="L65" s="3" t="inlineStr">
         <is>
           <t>שניהם</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>מומלץ להגיע רגוע ולעדכן את המטפל/ת על שבוע ההריון ועל כל רגישות. ההתאמה האישית תאושר על ידי הצוות.</t>
+        </is>
+      </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>מומלץ לשתות הרבה מים לאחר העיסוי, לנוח ולהימנע ממאמץ גופני אינטנסיבי באותו יום.</t>
+        </is>
+      </c>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>אין זמן החלמה — ניתן לחזור לשגרה מיד.</t>
+        </is>
+      </c>
+      <c r="P65" t="inlineStr">
+        <is>
+          <t>עדין ומותאם לנשים בהריון.</t>
+        </is>
+      </c>
+      <c r="Q65" t="inlineStr">
+        <is>
+          <t>ניתן כטיפול בודד או קבוע לאורך ההריון, בהתאם להתאמה אישית.</t>
+        </is>
+      </c>
+      <c r="R65" t="inlineStr">
+        <is>
+          <t>תחושת ההרפיה מורגשת מיד; לתחזוקה מתמשכת מומלץ עיסוי קבוע.</t>
+        </is>
+      </c>
+      <c r="S65" t="inlineStr">
+        <is>
+          <t>עיסוי עדין המותאם לנשים בהריון לשחרור מתחים ולשיפור תחושת הרווחה, בליווי מטפל/ת מוסמך/ת.</t>
         </is>
       </c>
     </row>
@@ -4113,6 +5198,41 @@
           <t>שניהם - יתכן וזהה ל'עיסוי משולב/רפואי' מהמחירון</t>
         </is>
       </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>מומלץ להגיע רגוע, להימנע מארוחה כבדה כשעה לפני הטיפול, ולעדכן את המטפל/ת על אזורים רגישים או כאב.</t>
+        </is>
+      </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>מומלץ לשתות הרבה מים לאחר העיסוי, לנוח ולהימנע ממאמץ גופני אינטנסיבי באותו יום.</t>
+        </is>
+      </c>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>אין זמן החלמה — ניתן לחזור לשגרה מיד.</t>
+        </is>
+      </c>
+      <c r="P66" t="inlineStr">
+        <is>
+          <t>מותאם אישית לעוצמה המבוקשת.</t>
+        </is>
+      </c>
+      <c r="Q66" t="inlineStr">
+        <is>
+          <t>ניתן כטיפול בודד או כסדרה לתחזוקה לפי הצורך.</t>
+        </is>
+      </c>
+      <c r="R66" t="inlineStr">
+        <is>
+          <t>תחושת ההרפיה מורגשת מיד; לתחזוקה מתמשכת מומלץ עיסוי קבוע.</t>
+        </is>
+      </c>
+      <c r="S66" t="inlineStr">
+        <is>
+          <t>עיסוי משולב המשלב מספר טכניקות המותאמות אישית לצרכים שלך.</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
@@ -4159,6 +5279,41 @@
           <t>שניהם</t>
         </is>
       </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>מומלץ להגיע רגוע, להימנע מארוחה כבדה כשעה לפני הטיפול, ולעדכן את המטפל/ת על אזורים רגישים או כאב.</t>
+        </is>
+      </c>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>מומלץ לשתות הרבה מים לאחר העיסוי, לנוח ולהימנע ממאמץ גופני אינטנסיבי באותו יום.</t>
+        </is>
+      </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>אין זמן החלמה — ניתן לחזור לשגרה מיד.</t>
+        </is>
+      </c>
+      <c r="P67" t="inlineStr">
+        <is>
+          <t>לחץ בינוני ומרגיע; ניתן להתאים את העוצמה מול המטפל/ת.</t>
+        </is>
+      </c>
+      <c r="Q67" t="inlineStr">
+        <is>
+          <t>ניתן כטיפול בודד או כסדרה לתחזוקה לפי הצורך.</t>
+        </is>
+      </c>
+      <c r="R67" t="inlineStr">
+        <is>
+          <t>תחושת ההרפיה מורגשת מיד; לתחזוקה מתמשכת מומלץ עיסוי קבוע.</t>
+        </is>
+      </c>
+      <c r="S67" t="inlineStr">
+        <is>
+          <t>רפלקסולוגיה — לחיצות בנקודות בכפות הרגליים והידיים לאיזון ולשיפור בריאות כללית.</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
@@ -4247,6 +5402,41 @@
       <c r="L69" s="3" t="inlineStr">
         <is>
           <t>מחירון בלבד</t>
+        </is>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>מומלץ להגיע רגוע, להימנע מארוחה כבדה כשעה לפני הטיפול, ולעדכן את המטפל/ת על אזורים רגישים או כאב.</t>
+        </is>
+      </c>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>מומלץ לשתות הרבה מים לאחר העיסוי, לנוח ולהימנע ממאמץ גופני אינטנסיבי באותו יום.</t>
+        </is>
+      </c>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t>אין זמן החלמה — ניתן לחזור לשגרה מיד.</t>
+        </is>
+      </c>
+      <c r="P69" t="inlineStr">
+        <is>
+          <t>עדין מאוד — לחץ קל.</t>
+        </is>
+      </c>
+      <c r="Q69" t="inlineStr">
+        <is>
+          <t>ניתן כטיפול בודד או כסדרה לתחזוקה לפי הצורך.</t>
+        </is>
+      </c>
+      <c r="R69" t="inlineStr">
+        <is>
+          <t>תחושת ההרפיה מורגשת מיד; לתחזוקה מתמשכת מומלץ עיסוי קבוע.</t>
+        </is>
+      </c>
+      <c r="S69" t="inlineStr">
+        <is>
+          <t>עיסוי לימפטי עדין לעידוד ניקוז לימפטי ושיפור זרימת הדם.</t>
         </is>
       </c>
     </row>
@@ -4291,6 +5481,41 @@
           <t>מחירון בלבד</t>
         </is>
       </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>מומלץ להגיע רגוע, להימנע מארוחה כבדה כשעה לפני הטיפול, ולעדכן את המטפל/ת על אזורים רגישים או כאב.</t>
+        </is>
+      </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>מומלץ לשתות הרבה מים לאחר העיסוי, לנוח ולהימנע ממאמץ גופני אינטנסיבי באותו יום.</t>
+        </is>
+      </c>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t>ייתכן אודם/סימנים זמניים באזור החולפים תוך ימים.</t>
+        </is>
+      </c>
+      <c r="P70" t="inlineStr">
+        <is>
+          <t>ייתכן תחושת לחץ/משיכה; ייתכן אודם זמני באזור.</t>
+        </is>
+      </c>
+      <c r="Q70" t="inlineStr">
+        <is>
+          <t>ניתן כטיפול בודד או כסדרה לתחזוקה לפי הצורך.</t>
+        </is>
+      </c>
+      <c r="R70" t="inlineStr">
+        <is>
+          <t>תחושת ההרפיה מורגשת מיד; לתחזוקה מתמשכת מומלץ עיסוי קבוע.</t>
+        </is>
+      </c>
+      <c r="S70" t="inlineStr">
+        <is>
+          <t>חיג'אמה (הקזת דם) לניקוי הגוף ושיפור זרימת הדם.</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
@@ -4331,6 +5556,41 @@
       <c r="L71" s="3" t="inlineStr">
         <is>
           <t>מחירון בלבד</t>
+        </is>
+      </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>מומלץ להגיע רגוע, להימנע מארוחה כבדה כשעה לפני הטיפול, ולעדכן את המטפל/ת על אזורים רגישים או כאב.</t>
+        </is>
+      </c>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>מומלץ לשתות הרבה מים לאחר העיסוי, לנוח ולהימנע ממאמץ גופני אינטנסיבי באותו יום.</t>
+        </is>
+      </c>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>ייתכן אודם/סימנים עגולים זמניים באזור החולפים תוך ימים.</t>
+        </is>
+      </c>
+      <c r="P71" t="inlineStr">
+        <is>
+          <t>ייתכן תחושת לחץ/משיכה; ייתכן אודם זמני באזור.</t>
+        </is>
+      </c>
+      <c r="Q71" t="inlineStr">
+        <is>
+          <t>ניתן כטיפול בודד או כסדרה לתחזוקה לפי הצורך.</t>
+        </is>
+      </c>
+      <c r="R71" t="inlineStr">
+        <is>
+          <t>תחושת ההרפיה מורגשת מיד; לתחזוקה מתמשכת מומלץ עיסוי קבוע.</t>
+        </is>
+      </c>
+      <c r="S71" t="inlineStr">
+        <is>
+          <t>כוסות רוח לשחרור ולשיפור זרימת הדם באזורים ממוקדים.</t>
         </is>
       </c>
     </row>
@@ -5321,6 +6581,41 @@
           <t>אתר</t>
         </is>
       </c>
+      <c r="M97" t="inlineStr">
+        <is>
+          <t>מומלץ להימנע מקפאין וממדללי דם ביום הטיפול ולהגיע ללא איפור באזור המטופל. מומלצת פגישת ייעוץ מקדימה.</t>
+        </is>
+      </c>
+      <c r="N97" t="inlineStr">
+        <is>
+          <t>יש לשמור על האזור נקי ויבש, להימנע מחשיפה לשמש, סאונה ובריכה, ולמרוח משחה מרגיעה לפי הנחיית המטפל/ת בימי ההחלמה.</t>
+        </is>
+      </c>
+      <c r="O97" t="inlineStr">
+        <is>
+          <t>ההחלמה נמשכת מספר ימים עד כשבועיים; ייתכנו אודם או קילופים קלים באזור.</t>
+        </is>
+      </c>
+      <c r="P97" t="inlineStr">
+        <is>
+          <t>אי-נוחות קלה; נעשה שימוש בחומר הרדמה מקומי לנוחות.</t>
+        </is>
+      </c>
+      <c r="Q97" t="inlineStr">
+        <is>
+          <t>עד 2 טיפולים כולל השלמת צבע; מומלצת פגישת ייעוץ תחילה.</t>
+        </is>
+      </c>
+      <c r="R97" t="inlineStr">
+        <is>
+          <t>נשמר לאורך זמן (חודשים עד שנים) בהתאם לסוג העור ולתחזוקה.</t>
+        </is>
+      </c>
+      <c r="S97" t="inlineStr">
+        <is>
+          <t>הדמיית שיער בעזרת מחט עדינה המציירת שערות; מתאים בעיקר לעור יבש.</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="3" t="inlineStr">
@@ -5367,6 +6662,41 @@
           <t>אתר</t>
         </is>
       </c>
+      <c r="M98" t="inlineStr">
+        <is>
+          <t>מומלץ להימנע מקפאין וממדללי דם ביום הטיפול ולהגיע ללא איפור באזור המטופל. מומלצת פגישת ייעוץ מקדימה.</t>
+        </is>
+      </c>
+      <c r="N98" t="inlineStr">
+        <is>
+          <t>יש לשמור על האזור נקי ויבש, להימנע מחשיפה לשמש, סאונה ובריכה, ולמרוח משחה מרגיעה לפי הנחיית המטפל/ת בימי ההחלמה.</t>
+        </is>
+      </c>
+      <c r="O98" t="inlineStr">
+        <is>
+          <t>ההחלמה נמשכת מספר ימים עד כשבועיים; ייתכנו אודם או קילופים קלים באזור.</t>
+        </is>
+      </c>
+      <c r="P98" t="inlineStr">
+        <is>
+          <t>אי-נוחות קלה; נעשה שימוש בחומר הרדמה מקומי לנוחות.</t>
+        </is>
+      </c>
+      <c r="Q98" t="inlineStr">
+        <is>
+          <t>עד 2 טיפולים כולל השלמת צבע; מומלצת פגישת ייעוץ תחילה.</t>
+        </is>
+      </c>
+      <c r="R98" t="inlineStr">
+        <is>
+          <t>נשמר לאורך זמן (חודשים עד שנים) בהתאם לסוג העור ולתחזוקה.</t>
+        </is>
+      </c>
+      <c r="S98" t="inlineStr">
+        <is>
+          <t>שיטת הפודרה (פיקסלים) ליצירת שכבות עדינות למראה טבעי; מתאים לכל סוגי העור.</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="3" t="inlineStr">
@@ -5413,6 +6743,41 @@
           <t>אתר</t>
         </is>
       </c>
+      <c r="M99" t="inlineStr">
+        <is>
+          <t>מומלץ להימנע מקפאין וממדללי דם ביום הטיפול ולהגיע ללא איפור באזור המטופל. מומלצת פגישת ייעוץ מקדימה.</t>
+        </is>
+      </c>
+      <c r="N99" t="inlineStr">
+        <is>
+          <t>יש לשמור על האזור נקי ויבש, להימנע מחשיפה לשמש, סאונה ובריכה, ולמרוח משחה מרגיעה לפי הנחיית המטפל/ת בימי ההחלמה.</t>
+        </is>
+      </c>
+      <c r="O99" t="inlineStr">
+        <is>
+          <t>ההחלמה נמשכת מספר ימים עד כשבועיים; ייתכנו אודם או קילופים קלים באזור.</t>
+        </is>
+      </c>
+      <c r="P99" t="inlineStr">
+        <is>
+          <t>אי-נוחות קלה; נעשה שימוש בחומר הרדמה מקומי לנוחות.</t>
+        </is>
+      </c>
+      <c r="Q99" t="inlineStr">
+        <is>
+          <t>עד 2 טיפולים כולל השלמת צבע; מומלצת פגישת ייעוץ תחילה.</t>
+        </is>
+      </c>
+      <c r="R99" t="inlineStr">
+        <is>
+          <t>נשמר לאורך זמן (חודשים עד שנים) בהתאם לסוג העור ולתחזוקה.</t>
+        </is>
+      </c>
+      <c r="S99" t="inlineStr">
+        <is>
+          <t>שיטה משולבת של הצללה/פודרה עם שיטת השערה; מתאים לכל סוגי העור.</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="3" t="inlineStr">
@@ -5459,6 +6824,41 @@
           <t>אתר</t>
         </is>
       </c>
+      <c r="M100" t="inlineStr">
+        <is>
+          <t>מומלץ להימנע מקפאין וממדללי דם ביום הטיפול ולהגיע ללא איפור באזור המטופל. מומלצת פגישת ייעוץ מקדימה.</t>
+        </is>
+      </c>
+      <c r="N100" t="inlineStr">
+        <is>
+          <t>יש לשמור על האזור נקי ויבש, להימנע מחשיפה לשמש, סאונה ובריכה, ולמרוח משחה מרגיעה לפי הנחיית המטפל/ת בימי ההחלמה.</t>
+        </is>
+      </c>
+      <c r="O100" t="inlineStr">
+        <is>
+          <t>ההחלמה נמשכת מספר ימים עד כשבועיים; ייתכנו אודם או קילופים קלים באזור.</t>
+        </is>
+      </c>
+      <c r="P100" t="inlineStr">
+        <is>
+          <t>אי-נוחות קלה; נעשה שימוש בחומר הרדמה מקומי לנוחות.</t>
+        </is>
+      </c>
+      <c r="Q100" t="inlineStr">
+        <is>
+          <t>עד 2 טיפולים כולל השלמת צבע; מומלצת פגישת ייעוץ תחילה.</t>
+        </is>
+      </c>
+      <c r="R100" t="inlineStr">
+        <is>
+          <t>נשמר לאורך זמן (חודשים עד שנים) בהתאם לסוג העור ולתחזוקה.</t>
+        </is>
+      </c>
+      <c r="S100" t="inlineStr">
+        <is>
+          <t>תיחום קו הריסים התחתון בטכניקה מתקדמת ועדינה.</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
@@ -5505,6 +6905,41 @@
           <t>אתר</t>
         </is>
       </c>
+      <c r="M101" t="inlineStr">
+        <is>
+          <t>מומלץ להימנע מקפאין וממדללי דם ביום הטיפול ולהגיע ללא איפור באזור המטופל. מומלצת פגישת ייעוץ מקדימה.</t>
+        </is>
+      </c>
+      <c r="N101" t="inlineStr">
+        <is>
+          <t>יש לשמור על האזור נקי ויבש, להימנע מחשיפה לשמש, סאונה ובריכה, ולמרוח משחה מרגיעה לפי הנחיית המטפל/ת בימי ההחלמה.</t>
+        </is>
+      </c>
+      <c r="O101" t="inlineStr">
+        <is>
+          <t>ההחלמה נמשכת מספר ימים עד כשבועיים; ייתכנו אודם או קילופים קלים באזור.</t>
+        </is>
+      </c>
+      <c r="P101" t="inlineStr">
+        <is>
+          <t>אי-נוחות קלה; נעשה שימוש בחומר הרדמה מקומי לנוחות.</t>
+        </is>
+      </c>
+      <c r="Q101" t="inlineStr">
+        <is>
+          <t>עד 2 טיפולים כולל השלמת צבע; מומלצת פגישת ייעוץ תחילה.</t>
+        </is>
+      </c>
+      <c r="R101" t="inlineStr">
+        <is>
+          <t>נשמר לאורך זמן (חודשים עד שנים) בהתאם לסוג העור ולתחזוקה.</t>
+        </is>
+      </c>
+      <c r="S101" t="inlineStr">
+        <is>
+          <t>תיחום קו הריסים העליון בטכניקה מתקדמת ועדינה.</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="3" t="inlineStr">
@@ -5551,6 +6986,41 @@
           <t>אתר</t>
         </is>
       </c>
+      <c r="M102" t="inlineStr">
+        <is>
+          <t>מומלץ להימנע מקפאין וממדללי דם ביום הטיפול ולהגיע ללא איפור באזור המטופל. מומלצת פגישת ייעוץ מקדימה.</t>
+        </is>
+      </c>
+      <c r="N102" t="inlineStr">
+        <is>
+          <t>יש לשמור על האזור נקי ויבש, להימנע מחשיפה לשמש, סאונה ובריכה, ולמרוח משחה מרגיעה לפי הנחיית המטפל/ת בימי ההחלמה.</t>
+        </is>
+      </c>
+      <c r="O102" t="inlineStr">
+        <is>
+          <t>ההחלמה נמשכת מספר ימים עד כשבועיים; ייתכנו אודם או קילופים קלים באזור.</t>
+        </is>
+      </c>
+      <c r="P102" t="inlineStr">
+        <is>
+          <t>אי-נוחות קלה; נעשה שימוש בחומר הרדמה מקומי לנוחות.</t>
+        </is>
+      </c>
+      <c r="Q102" t="inlineStr">
+        <is>
+          <t>עד 2 טיפולים כולל השלמת צבע; מומלצת פגישת ייעוץ תחילה.</t>
+        </is>
+      </c>
+      <c r="R102" t="inlineStr">
+        <is>
+          <t>נשמר לאורך זמן (חודשים עד שנים) בהתאם לסוג העור ולתחזוקה.</t>
+        </is>
+      </c>
+      <c r="S102" t="inlineStr">
+        <is>
+          <t>אייליינר עליון בטכניקה מתקדמת למראה מוגדר.</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="3" t="inlineStr">
@@ -5597,6 +7067,41 @@
           <t>אתר</t>
         </is>
       </c>
+      <c r="M103" t="inlineStr">
+        <is>
+          <t>מומלץ להימנע מקפאין וממדללי דם ביום הטיפול ולהגיע ללא איפור באזור המטופל. מומלצת פגישת ייעוץ מקדימה.</t>
+        </is>
+      </c>
+      <c r="N103" t="inlineStr">
+        <is>
+          <t>יש לשמור על האזור נקי ויבש, להימנע מחשיפה לשמש, סאונה ובריכה, ולמרוח משחה מרגיעה לפי הנחיית המטפל/ת בימי ההחלמה.</t>
+        </is>
+      </c>
+      <c r="O103" t="inlineStr">
+        <is>
+          <t>ההחלמה נמשכת מספר ימים עד כשבועיים; ייתכנו אודם או קילופים קלים באזור.</t>
+        </is>
+      </c>
+      <c r="P103" t="inlineStr">
+        <is>
+          <t>אי-נוחות קלה; נעשה שימוש בחומר הרדמה מקומי לנוחות.</t>
+        </is>
+      </c>
+      <c r="Q103" t="inlineStr">
+        <is>
+          <t>עד 2 טיפולים כולל השלמת צבע; מומלצת פגישת ייעוץ תחילה.</t>
+        </is>
+      </c>
+      <c r="R103" t="inlineStr">
+        <is>
+          <t>נשמר לאורך זמן (חודשים עד שנים) בהתאם לסוג העור ולתחזוקה.</t>
+        </is>
+      </c>
+      <c r="S103" t="inlineStr">
+        <is>
+          <t>תיחום שפתיים בקו טבעי בטכניקה מתקדמת.</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="3" t="inlineStr">
@@ -5643,6 +7148,41 @@
           <t>אתר</t>
         </is>
       </c>
+      <c r="M104" t="inlineStr">
+        <is>
+          <t>מומלץ להימנע מקפאין וממדללי דם ביום הטיפול ולהגיע ללא איפור באזור המטופל. מומלצת פגישת ייעוץ מקדימה.</t>
+        </is>
+      </c>
+      <c r="N104" t="inlineStr">
+        <is>
+          <t>יש לשמור על האזור נקי ויבש, להימנע מחשיפה לשמש, סאונה ובריכה, ולמרוח משחה מרגיעה לפי הנחיית המטפל/ת בימי ההחלמה.</t>
+        </is>
+      </c>
+      <c r="O104" t="inlineStr">
+        <is>
+          <t>ההחלמה נמשכת מספר ימים עד כשבועיים; ייתכנו אודם או קילופים קלים באזור.</t>
+        </is>
+      </c>
+      <c r="P104" t="inlineStr">
+        <is>
+          <t>אי-נוחות קלה; נעשה שימוש בחומר הרדמה מקומי לנוחות.</t>
+        </is>
+      </c>
+      <c r="Q104" t="inlineStr">
+        <is>
+          <t>עד 2 טיפולים כולל השלמת צבע; מומלצת פגישת ייעוץ תחילה.</t>
+        </is>
+      </c>
+      <c r="R104" t="inlineStr">
+        <is>
+          <t>נשמר לאורך זמן (חודשים עד שנים) בהתאם לסוג העור ולתחזוקה.</t>
+        </is>
+      </c>
+      <c r="S104" t="inlineStr">
+        <is>
+          <t>מילוי שפתיים ותיחום למראה מלא וטבעי.</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="3" t="inlineStr">
@@ -5689,6 +7229,41 @@
           <t>אתר</t>
         </is>
       </c>
+      <c r="M105" t="inlineStr">
+        <is>
+          <t>מומלץ להימנע מקפאין וממדללי דם ביום הטיפול ולהגיע ללא איפור באזור המטופל. מומלצת פגישת ייעוץ מקדימה.</t>
+        </is>
+      </c>
+      <c r="N105" t="inlineStr">
+        <is>
+          <t>יש לשמור על האזור נקי ויבש, להימנע מחשיפה לשמש, סאונה ובריכה, ולמרוח משחה מרגיעה לפי הנחיית המטפל/ת בימי ההחלמה.</t>
+        </is>
+      </c>
+      <c r="O105" t="inlineStr">
+        <is>
+          <t>ההחלמה נמשכת מספר ימים עד כשבועיים; ייתכנו אודם או קילופים קלים באזור.</t>
+        </is>
+      </c>
+      <c r="P105" t="inlineStr">
+        <is>
+          <t>אי-נוחות קלה; נעשה שימוש בחומר הרדמה מקומי לנוחות.</t>
+        </is>
+      </c>
+      <c r="Q105" t="inlineStr">
+        <is>
+          <t>עד 2 טיפולים כולל השלמת צבע; מומלצת פגישת ייעוץ תחילה.</t>
+        </is>
+      </c>
+      <c r="R105" t="inlineStr">
+        <is>
+          <t>נשמר לאורך זמן (חודשים עד שנים) בהתאם לסוג העור ולתחזוקה.</t>
+        </is>
+      </c>
+      <c r="S105" t="inlineStr">
+        <is>
+          <t>מילוי קרקפת לנשים למראה מלא יותר, בטיפול של כשעה.</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="3" t="inlineStr">
@@ -5733,6 +7308,41 @@
       <c r="L106" s="3" t="inlineStr">
         <is>
           <t>אתר</t>
+        </is>
+      </c>
+      <c r="M106" t="inlineStr">
+        <is>
+          <t>מומלץ להימנע מקפאין וממדללי דם ביום הטיפול ולהגיע ללא איפור באזור המטופל. מומלצת פגישת ייעוץ מקדימה.</t>
+        </is>
+      </c>
+      <c r="N106" t="inlineStr">
+        <is>
+          <t>יש לשמור על האזור נקי ויבש, להימנע מחשיפה לשמש, סאונה ובריכה, ולמרוח משחה מרגיעה לפי הנחיית המטפל/ת בימי ההחלמה.</t>
+        </is>
+      </c>
+      <c r="O106" t="inlineStr">
+        <is>
+          <t>ההחלמה נמשכת מספר ימים עד כשבועיים; ייתכנו אודם או קילופים קלים באזור.</t>
+        </is>
+      </c>
+      <c r="P106" t="inlineStr">
+        <is>
+          <t>אי-נוחות קלה; נעשה שימוש בחומר הרדמה מקומי לנוחות.</t>
+        </is>
+      </c>
+      <c r="Q106" t="inlineStr">
+        <is>
+          <t>עד 2 טיפולים כולל השלמת צבע; מומלצת פגישת ייעוץ תחילה.</t>
+        </is>
+      </c>
+      <c r="R106" t="inlineStr">
+        <is>
+          <t>נשמר לאורך זמן (חודשים עד שנים) בהתאם לסוג העור ולתחזוקה.</t>
+        </is>
+      </c>
+      <c r="S106" t="inlineStr">
+        <is>
+          <t>מילוי קרקפת לגברים למראה מלא יותר, בטיפול של כשעה.</t>
         </is>
       </c>
     </row>
@@ -10261,7 +11871,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10700,6 +12310,330 @@
       <c r="E16" s="3" t="inlineStr">
         <is>
           <t>לתאם תור, איך יוצרים קשר, מספר טלפון</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>FAQ-16</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>האם צריך לקבוע תור מראש?</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>מומלץ לתאם תור מראש כדי להבטיח את הזמינות הרצויה. ניתן לתאם בטלפון *3691 או בהודעת ווטסאפ.</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>צריך תור מראש, אפשר להגיע בלי תור, walk in, هل احتاج موعد مسبق, بدون موعد</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>FAQ-17</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>CAT-03</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>כיצד כדאי להתכונן לטיפול פנים?</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>מומלץ להגיע ללא איפור ולהימנע מחומצות, רטינול או פילינג ביתי מספר ימים לפני הטיפול. לפני טיפולים מבוססי אור יש להימנע מחשיפה ממושכת לשמש ומשיזוף.</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>איך להתכונן לטיפול פנים, מה לעשות לפני ניקוי פנים, הכנה לטיפול פנים, كيف أستعد لتنظيف البشرة, تحضير قبل علاج الوجه</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>FAQ-18</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>CAT-03</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>מה מומלץ לעשות אחרי טיפול פנים?</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>מומלץ להימנע מאיפור למשך מספר שעות, להקפיד על קרם הגנה SPF, ולהימנע מחשיפה ישירה לשמש, מסאונה וממאמץ מזיע ביום-יומיים הראשונים.</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>מה לעשות אחרי טיפול פנים, טיפוח אחרי ניקוי פנים, אחרי פילינג פנים, ماذا أفعل بعد علاج الوجه, العناية بعد تنظيف البشرة</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>FAQ-19</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>CAT-03</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>האם טיפול פנים כואב?</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>רוב טיפולי הפנים נעימים; ייתכן אי-נוחות קלה בשלב ניקוז הקומדונים או תחושת חום/עקצוץ קלה בטיפולים טכנולוגיים, שחולפת במהירות.</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>טיפול פנים כואב, זה כואב ניקוי פנים, האם ניקוי עמוק כואב, هل علاج الوجه مؤلم, تنظيف البشرة يوجع</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>FAQ-20</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>CAT-04</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>מה כדאי ללבוש או להביא לעיסוי?</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>אין צורך בהכנה מיוחדת — מגיעים בבגדים נוחים והמטפל/ת ידאג/תדאג לפרטיות ולנוחות. מומלץ לעדכן מראש על אזורים רגישים או כאב.</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>מה ללבוש לעיסוי, מה להביא לעיסוי, איך מגיעים לעיסוי, ماذا ألبس للمساج, ماذا أحضر للمساج</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>FAQ-21</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>CAT-04</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>האם כדאי לאכול לפני עיסוי?</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>מומלץ להימנע מארוחה כבדה כשעה לפני העיסוי ולהגיע רגוע. כדאי לשתות מים לפני ואחרי הטיפול.</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>לאכול לפני עיסוי, ארוחה לפני עיסוי, هل آكل قبل المساج, الأكل قبل المساج</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>FAQ-22</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>CAT-01</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>כמה זמן מחזיק לק ג'ל?</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>לק ג'ל נשמר בדרך כלל כשבועיים-שלושה בהתאם לקצב צמיחת הציפורן ולתחזוקה. מומלץ ריענון כל 2-3 שבועות.</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>כמה מחזיק לק גל, לק ג'ל כמה זמן, כמה זמן נשאר לק גל, كم يدوم الجل, مدة طلاء الجل</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>FAQ-23</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>CAT-07</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>כמה זמן נשמר איפור קבוע / עיצוב גבות?</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>התוצאה נשמרת לאורך זמן (חודשים עד שנים) בהתאם לסוג העור ולתחזוקה. לרוב מומלצת השלמת צבע במסגרת עד 2 טיפולים.</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>כמה זמן נשאר איפור קבוע, כמה מחזיק מיקרובליידינג, גבות קבועות כמה זמן, كم يدوم التاتو, مدة الحواجب الدائمة</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>FAQ-24</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>CAT-07</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>איך נראה תהליך ההחלמה אחרי איפור קבוע?</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>ההחלמה נמשכת מספר ימים עד כשבועיים; ייתכנו אודם או קילופים קלים. יש לשמור על האזור נקי ויבש ולהימנע מחשיפה לשמש, סאונה ובריכה בימי ההחלמה.</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>החלמה אחרי איפור קבוע, אחרי מיקרובליידינג, כמה זמן ההחלמה של גבות, تعافي بعد التاتو, شفاء الحواجب الدائمة</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>FAQ-25</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>האם אתם מטפלים גם בגברים?</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>בהחלט! יש לנו טיפולים לגברים, בהם טיפול פנים לגבר (Man T), תספורת ועיצוב זקן, עיסויים ומילוי קרקפת לגבר.</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>יש טיפולים לגברים, אתם מקבלים גברים, טיפול פנים לגבר, هل تستقبلون رجال, علاجات للرجال</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>FAQ-26</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>כמה זמן לפני אירוע כדאי לעשות טיפול פנים?</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>לטיפולי זוהר והחדרת לחות ניתן להגיע ממש סמוך לאירוע. לטיפולים עמוקים או טכנולוגיים מומלץ להקדים מספר ימים כדי לאפשר לעור להירגע. הצוות ישמח להמליץ על התזמון המתאים.</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>מתי לעשות טיפול פנים לפני אירוע, טיפול פנים לפני חתונה, כמה זמן לפני האירוע, متى أعمل علاج الوجه قبل المناسبة, تنظيف البشرة قبل العرس</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>FAQ-27</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>CAT-04</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>האם אפשר לקבל עיסוי בזמן הריון?</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>יש לנו עיסוי המותאם במיוחד לנשים בהריון, המבוצע על ידי מטפל/ת מוסמך/ת ומנוסה. לגבי התאמה אישית ובטיחות בשלב ההריון שלך, הצוות שלנו ישמח לאשר עבורך ב-*3691.</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>עיסוי בהריון, אפשר עיסוי כשבהריון, עיסוי לנשים בהריון, هل يجوز المساج للحامل, مساج للحامل</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: fix chatbot backend and frontend integration
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/MeDay_Treatments_Data_finalalmost.xlsx
+++ b/backend/MeDay_Treatments_Data_finalalmost.xlsx
@@ -932,7 +932,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -968,6 +968,11 @@
           <t>data_source</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>short_description</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -989,6 +994,11 @@
           <t>אתר + מחירון</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>טיפוח מקצועי לציפורניים ולכפות הידיים והרגליים — מניקור, פדיקור, בנייה ועיצוב.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -1010,6 +1020,11 @@
           <t>מחירון בלבד - האתר ריק בקטגוריה זו</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>תספורות, צבע, החלקות, טיפולי שיקום ועיצוב שיער לנשים, גברים וילדים.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -1035,6 +1050,11 @@
           <t>אתר + מחירון</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>טיפולי פנים לניקוי, חידוש והזנת העור — מטיפולים קלאסיים ועד טכנולוגיים מתקדמים.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -1060,6 +1080,11 @@
           <t>אתר + מחירון</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>מגוון עיסויים וטיפולי גוף להרפיה, שחרור מתחים ושיפור תחושת הרווחה.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -1081,6 +1106,11 @@
           <t>מחירון בלבד - האתר ריק בקטגוריה זו</t>
         </is>
       </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>הסרת שיער לאזורי הגוף והפנים בטיפול מקצועי.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -1102,6 +1132,11 @@
           <t>מחירון בלבד - האתר ריק בקטגוריה זו</t>
         </is>
       </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>איפור מקצועי לאירועים, לכלות וליום-יום, בהתאמה אישית.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -1123,6 +1158,11 @@
           <t>אתר + מחירון</t>
         </is>
       </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>איפור קבוע ועיצוב גבות, ריסים ושפתיים למראה מוגדר וטבעי לאורך זמן.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -1144,6 +1184,11 @@
           <t>אתר בלבד</t>
         </is>
       </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>מפגשי ייעוץ אישי לפיתוח סטייל, התאמת מלתחה ואביזור.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -1163,6 +1208,11 @@
       <c r="E10" s="3" t="inlineStr">
         <is>
           <t>מחירון בלבד - האתר ריק בקטגוריה זו</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>טיפולי אסתטיקה מתקדמים בהתאמה אישית. הצוות המקצועי ישמח לייעץ ולהתאים עבורך.</t>
         </is>
       </c>
     </row>
@@ -1784,7 +1834,11 @@
           <t>פדיקור אסתטי כולל הסרת לק ג'ל</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr"/>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>טיפול פדיקור לטיפוח כפות הרגליים והציפורניים.</t>
+        </is>
+      </c>
       <c r="F8" s="3" t="inlineStr"/>
       <c r="G8" s="3" t="inlineStr"/>
       <c r="H8" s="3" t="inlineStr"/>
@@ -1822,7 +1876,11 @@
           <t>פדיקור פרא-רפואי</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr"/>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>טיפול פדיקור לטיפוח כפות הרגליים והציפורניים.</t>
+        </is>
+      </c>
       <c r="F9" s="3" t="inlineStr"/>
       <c r="G9" s="3" t="inlineStr"/>
       <c r="H9" s="3" t="inlineStr"/>
@@ -1860,7 +1918,11 @@
           <t>פדיקור טיפולי (עצמאי)</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr"/>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>טיפול פדיקור לטיפוח כפות הרגליים והציפורניים.</t>
+        </is>
+      </c>
       <c r="F10" s="3" t="inlineStr"/>
       <c r="G10" s="3" t="inlineStr"/>
       <c r="H10" s="3" t="inlineStr"/>
@@ -1898,7 +1960,11 @@
           <t>מניקור לק ג'ל תיקון מבנה אנטומי</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>טיפול מניקור לטיפוח, ניקוי ועיצוב הציפורניים.</t>
+        </is>
+      </c>
       <c r="F11" s="3" t="inlineStr"/>
       <c r="G11" s="3" t="inlineStr"/>
       <c r="H11" s="3" t="n">
@@ -1938,7 +2004,11 @@
           <t>הסרת לק ג'ל + מניקור</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr"/>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>טיפול מניקור לטיפוח, ניקוי ועיצוב הציפורניים.</t>
+        </is>
+      </c>
       <c r="F12" s="3" t="inlineStr"/>
       <c r="G12" s="3" t="inlineStr"/>
       <c r="H12" s="3" t="n">
@@ -1978,7 +2048,11 @@
           <t>בנייה - אורך קצר-בינוני</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>טיפול בנייה או מילוי לעיצוב ולחיזוק הציפורניים.</t>
+        </is>
+      </c>
       <c r="F13" s="3" t="inlineStr"/>
       <c r="G13" s="3" t="inlineStr"/>
       <c r="H13" s="3" t="n">
@@ -2018,7 +2092,11 @@
           <t>בנייה - אורך מלא</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr"/>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>טיפול בנייה או מילוי לעיצוב ולחיזוק הציפורניים.</t>
+        </is>
+      </c>
       <c r="F14" s="3" t="inlineStr"/>
       <c r="G14" s="3" t="inlineStr"/>
       <c r="H14" s="3" t="n">
@@ -2058,7 +2136,11 @@
           <t>מילוי ללא בנייה - אורך קצר-בינוני</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>טיפול בנייה או מילוי לעיצוב ולחיזוק הציפורניים.</t>
+        </is>
+      </c>
       <c r="F15" s="3" t="inlineStr"/>
       <c r="G15" s="3" t="inlineStr"/>
       <c r="H15" s="3" t="n">
@@ -2098,7 +2180,11 @@
           <t>מילוי ללא בנייה - אורך מלא</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr"/>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>טיפול בנייה או מילוי לעיצוב ולחיזוק הציפורניים.</t>
+        </is>
+      </c>
       <c r="F16" s="3" t="inlineStr"/>
       <c r="G16" s="3" t="inlineStr"/>
       <c r="H16" s="3" t="n">
@@ -2138,7 +2224,11 @@
           <t>בנייה/תיקון ציפורן בודדת</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>טיפול בנייה או מילוי לעיצוב ולחיזוק הציפורניים.</t>
+        </is>
+      </c>
       <c r="F17" s="3" t="inlineStr"/>
       <c r="G17" s="3" t="inlineStr"/>
       <c r="H17" s="3" t="n">
@@ -2178,7 +2268,11 @@
           <t>הסרת בנייה + מניקור</t>
         </is>
       </c>
-      <c r="E18" s="3" t="inlineStr"/>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>טיפול בנייה או מילוי לעיצוב ולחיזוק הציפורניים.</t>
+        </is>
+      </c>
       <c r="F18" s="3" t="inlineStr"/>
       <c r="G18" s="3" t="inlineStr"/>
       <c r="H18" s="3" t="n">
@@ -2218,7 +2312,11 @@
           <t>פרנץ' קבוע</t>
         </is>
       </c>
-      <c r="E19" s="3" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>תוספת עיצוב וקישוט לציפורניים.</t>
+        </is>
+      </c>
       <c r="F19" s="3" t="inlineStr"/>
       <c r="G19" s="3" t="inlineStr"/>
       <c r="H19" s="3" t="n">
@@ -2258,7 +2356,11 @@
           <t>תוספת קישוטים</t>
         </is>
       </c>
-      <c r="E20" s="3" t="inlineStr"/>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>תוספת עיצוב וקישוט לציפורניים.</t>
+        </is>
+      </c>
       <c r="F20" s="3" t="inlineStr"/>
       <c r="G20" s="3" t="inlineStr"/>
       <c r="H20" s="3" t="n">
@@ -2298,7 +2400,11 @@
           <t>פרנץ'/אומברה</t>
         </is>
       </c>
-      <c r="E21" s="3" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>תוספת עיצוב וקישוט לציפורניים.</t>
+        </is>
+      </c>
       <c r="F21" s="3" t="inlineStr"/>
       <c r="G21" s="3" t="inlineStr"/>
       <c r="H21" s="3" t="n">
@@ -2338,7 +2444,11 @@
           <t>תספורת נשים</t>
         </is>
       </c>
-      <c r="E22" s="3" t="inlineStr"/>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>תספורת ועיצוב שיער.</t>
+        </is>
+      </c>
       <c r="F22" s="3" t="inlineStr"/>
       <c r="G22" s="3" t="inlineStr"/>
       <c r="H22" s="3" t="n">
@@ -2378,7 +2488,11 @@
           <t>צבע שורש</t>
         </is>
       </c>
-      <c r="E23" s="3" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>צביעת שיער ועיצוב גוון.</t>
+        </is>
+      </c>
       <c r="F23" s="3" t="inlineStr"/>
       <c r="G23" s="3" t="inlineStr"/>
       <c r="H23" s="3" t="n">
@@ -2418,7 +2532,11 @@
           <t>צבע מלא/שינוי גוון</t>
         </is>
       </c>
-      <c r="E24" s="3" t="inlineStr"/>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>צביעת שיער ועיצוב גוון.</t>
+        </is>
+      </c>
       <c r="F24" s="3" t="inlineStr"/>
       <c r="G24" s="3" t="inlineStr"/>
       <c r="H24" s="3" t="n">
@@ -2458,7 +2576,11 @@
           <t>שטיפה</t>
         </is>
       </c>
-      <c r="E25" s="3" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>צביעת שיער ועיצוב גוון.</t>
+        </is>
+      </c>
       <c r="F25" s="3" t="inlineStr"/>
       <c r="G25" s="3" t="inlineStr"/>
       <c r="H25" s="3" t="n">
@@ -2498,7 +2620,11 @@
           <t>גוונים חצי ראש</t>
         </is>
       </c>
-      <c r="E26" s="3" t="inlineStr"/>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>שירות עיצוב וטיפוח שיער.</t>
+        </is>
+      </c>
       <c r="F26" s="3" t="inlineStr"/>
       <c r="G26" s="3" t="inlineStr"/>
       <c r="H26" s="3" t="n">
@@ -2538,7 +2664,11 @@
           <t>גוונים ראש מלא</t>
         </is>
       </c>
-      <c r="E27" s="3" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>שירות עיצוב וטיפוח שיער.</t>
+        </is>
+      </c>
       <c r="F27" s="3" t="inlineStr"/>
       <c r="G27" s="3" t="inlineStr"/>
       <c r="H27" s="3" t="n">
@@ -2578,7 +2708,11 @@
           <t>גוונים ראש מלא - שיער צבוע</t>
         </is>
       </c>
-      <c r="E28" s="3" t="inlineStr"/>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>שירות עיצוב וטיפוח שיער.</t>
+        </is>
+      </c>
       <c r="F28" s="3" t="inlineStr"/>
       <c r="G28" s="3" t="inlineStr"/>
       <c r="H28" s="3" t="n">
@@ -2618,7 +2752,11 @@
           <t>פן קצר</t>
         </is>
       </c>
-      <c r="E29" s="3" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>פן ועיצוב שיער.</t>
+        </is>
+      </c>
       <c r="F29" s="3" t="inlineStr"/>
       <c r="G29" s="3" t="inlineStr"/>
       <c r="H29" s="3" t="n">
@@ -2658,7 +2796,11 @@
           <t>פן בינוני-ארוך</t>
         </is>
       </c>
-      <c r="E30" s="3" t="inlineStr"/>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>פן ועיצוב שיער.</t>
+        </is>
+      </c>
       <c r="F30" s="3" t="inlineStr"/>
       <c r="G30" s="3" t="inlineStr"/>
       <c r="H30" s="3" t="n">
@@ -2698,7 +2840,11 @@
           <t>פן מעוצב</t>
         </is>
       </c>
-      <c r="E31" s="3" t="inlineStr"/>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>פן ועיצוב שיער.</t>
+        </is>
+      </c>
       <c r="F31" s="3" t="inlineStr"/>
       <c r="G31" s="3" t="inlineStr"/>
       <c r="H31" s="3" t="n">
@@ -2738,7 +2884,11 @@
           <t>טיפול תלתלים - שיקום</t>
         </is>
       </c>
-      <c r="E32" s="3" t="inlineStr"/>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>טיפול לחיזוק, שיקום וטיפוח השיער.</t>
+        </is>
+      </c>
       <c r="F32" s="3" t="inlineStr"/>
       <c r="G32" s="3" t="inlineStr"/>
       <c r="H32" s="3" t="inlineStr"/>
@@ -2776,7 +2926,11 @@
           <t>תספורת פוני</t>
         </is>
       </c>
-      <c r="E33" s="3" t="inlineStr"/>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>תספורת ועיצוב שיער.</t>
+        </is>
+      </c>
       <c r="F33" s="3" t="inlineStr"/>
       <c r="G33" s="3" t="inlineStr"/>
       <c r="H33" s="3" t="n">
@@ -2816,7 +2970,11 @@
           <t>טיפול משקם לשיער</t>
         </is>
       </c>
-      <c r="E34" s="3" t="inlineStr"/>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>טיפול לחיזוק, שיקום וטיפוח השיער.</t>
+        </is>
+      </c>
       <c r="F34" s="3" t="inlineStr"/>
       <c r="G34" s="3" t="inlineStr"/>
       <c r="H34" s="3" t="inlineStr"/>
@@ -2854,7 +3012,11 @@
           <t>תספורת גברים</t>
         </is>
       </c>
-      <c r="E35" s="3" t="inlineStr"/>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>תספורת ועיצוב שיער.</t>
+        </is>
+      </c>
       <c r="F35" s="3" t="inlineStr"/>
       <c r="G35" s="3" t="inlineStr"/>
       <c r="H35" s="3" t="n">
@@ -2894,7 +3056,11 @@
           <t>עיצוב זקן + תספורת</t>
         </is>
       </c>
-      <c r="E36" s="3" t="inlineStr"/>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>תספורת ועיצוב שיער.</t>
+        </is>
+      </c>
       <c r="F36" s="3" t="inlineStr"/>
       <c r="G36" s="3" t="inlineStr"/>
       <c r="H36" s="3" t="n">
@@ -2934,7 +3100,11 @@
           <t>עיצוב וסידור זקן</t>
         </is>
       </c>
-      <c r="E37" s="3" t="inlineStr"/>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>עיצוב וטיפוח זקן.</t>
+        </is>
+      </c>
       <c r="F37" s="3" t="inlineStr"/>
       <c r="G37" s="3" t="inlineStr"/>
       <c r="H37" s="3" t="n">
@@ -2974,7 +3144,11 @@
           <t>שטיפת סילבר לגבר</t>
         </is>
       </c>
-      <c r="E38" s="3" t="inlineStr"/>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>צביעת שיער ועיצוב גוון.</t>
+        </is>
+      </c>
       <c r="F38" s="3" t="inlineStr"/>
       <c r="G38" s="3" t="inlineStr"/>
       <c r="H38" s="3" t="n">
@@ -3014,7 +3188,11 @@
           <t>גוונים לגבר</t>
         </is>
       </c>
-      <c r="E39" s="3" t="inlineStr"/>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>שירות עיצוב וטיפוח שיער.</t>
+        </is>
+      </c>
       <c r="F39" s="3" t="inlineStr"/>
       <c r="G39" s="3" t="inlineStr"/>
       <c r="H39" s="3" t="n">
@@ -3054,7 +3232,11 @@
           <t>תספורת ילדות</t>
         </is>
       </c>
-      <c r="E40" s="3" t="inlineStr"/>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>תספורת ועיצוב שיער.</t>
+        </is>
+      </c>
       <c r="F40" s="3" t="inlineStr"/>
       <c r="G40" s="3" t="inlineStr"/>
       <c r="H40" s="3" t="n">
@@ -3094,7 +3276,11 @@
           <t>תספורת ילד</t>
         </is>
       </c>
-      <c r="E41" s="3" t="inlineStr"/>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>תספורת ועיצוב שיער.</t>
+        </is>
+      </c>
       <c r="F41" s="3" t="inlineStr"/>
       <c r="G41" s="3" t="inlineStr"/>
       <c r="H41" s="3" t="n">
@@ -5336,7 +5522,11 @@
           <t>עיסוי קלאסי</t>
         </is>
       </c>
-      <c r="E68" s="3" t="inlineStr"/>
+      <c r="E68" s="3" t="inlineStr">
+        <is>
+          <t>עיסוי לטיפוח הגוף ולשיפור תחושת הרווחה (עיסוי קלאסי).</t>
+        </is>
+      </c>
       <c r="F68" s="3" t="inlineStr">
         <is>
           <t>הרפיה (קלאסי)</t>
@@ -5382,7 +5572,11 @@
           <t>עיסוי לימפטי</t>
         </is>
       </c>
-      <c r="E69" s="3" t="inlineStr"/>
+      <c r="E69" s="3" t="inlineStr">
+        <is>
+          <t>עיסוי לימפטי עדין לעידוד ניקוז לימפטי ושיפור זרימת הדם.</t>
+        </is>
+      </c>
       <c r="F69" s="3" t="inlineStr">
         <is>
           <t>ניקוז לימפטי, זרימת דם</t>
@@ -5461,7 +5655,11 @@
           <t>חיג'אמי - הקזת דם (ניקוי גוף)</t>
         </is>
       </c>
-      <c r="E70" s="3" t="inlineStr"/>
+      <c r="E70" s="3" t="inlineStr">
+        <is>
+          <t>חיג'אמה (הקזת דם) לניקוי הגוף ושיפור זרימת הדם.</t>
+        </is>
+      </c>
       <c r="F70" s="3" t="inlineStr">
         <is>
           <t>ניקוי גוף, זרימת דם</t>
@@ -5538,7 +5736,11 @@
           <t>כוסות רוח</t>
         </is>
       </c>
-      <c r="E71" s="3" t="inlineStr"/>
+      <c r="E71" s="3" t="inlineStr">
+        <is>
+          <t>כוסות רוח לשחרור ולשיפור זרימת הדם באזורים ממוקדים.</t>
+        </is>
+      </c>
       <c r="F71" s="3" t="inlineStr">
         <is>
           <t>זרימת דם, שחרור</t>
@@ -5615,7 +5817,11 @@
           <t>בית שחי</t>
         </is>
       </c>
-      <c r="E72" s="3" t="inlineStr"/>
+      <c r="E72" s="3" t="inlineStr">
+        <is>
+          <t>טיפול להסרת שיער באזור בית שחי.</t>
+        </is>
+      </c>
       <c r="F72" s="3" t="inlineStr"/>
       <c r="G72" s="3" t="inlineStr"/>
       <c r="H72" s="3" t="inlineStr"/>
@@ -5653,7 +5859,11 @@
           <t>ידיים חצי</t>
         </is>
       </c>
-      <c r="E73" s="3" t="inlineStr"/>
+      <c r="E73" s="3" t="inlineStr">
+        <is>
+          <t>טיפול להסרת שיער באזור ידיים חצי.</t>
+        </is>
+      </c>
       <c r="F73" s="3" t="inlineStr"/>
       <c r="G73" s="3" t="inlineStr"/>
       <c r="H73" s="3" t="inlineStr"/>
@@ -5691,7 +5901,11 @@
           <t>ידיים שלם</t>
         </is>
       </c>
-      <c r="E74" s="3" t="inlineStr"/>
+      <c r="E74" s="3" t="inlineStr">
+        <is>
+          <t>טיפול להסרת שיער באזור ידיים שלם.</t>
+        </is>
+      </c>
       <c r="F74" s="3" t="inlineStr"/>
       <c r="G74" s="3" t="inlineStr"/>
       <c r="H74" s="3" t="inlineStr"/>
@@ -5729,7 +5943,11 @@
           <t>רגליים חצי</t>
         </is>
       </c>
-      <c r="E75" s="3" t="inlineStr"/>
+      <c r="E75" s="3" t="inlineStr">
+        <is>
+          <t>טיפול להסרת שיער באזור רגליים חצי.</t>
+        </is>
+      </c>
       <c r="F75" s="3" t="inlineStr"/>
       <c r="G75" s="3" t="inlineStr"/>
       <c r="H75" s="3" t="inlineStr"/>
@@ -5767,7 +5985,11 @@
           <t>רגל שלמה</t>
         </is>
       </c>
-      <c r="E76" s="3" t="inlineStr"/>
+      <c r="E76" s="3" t="inlineStr">
+        <is>
+          <t>טיפול להסרת שיער באזור רגל שלמה.</t>
+        </is>
+      </c>
       <c r="F76" s="3" t="inlineStr"/>
       <c r="G76" s="3" t="inlineStr"/>
       <c r="H76" s="3" t="inlineStr"/>
@@ -5805,7 +6027,11 @@
           <t>מפשעות קו ביקיני</t>
         </is>
       </c>
-      <c r="E77" s="3" t="inlineStr"/>
+      <c r="E77" s="3" t="inlineStr">
+        <is>
+          <t>טיפול להסרת שיער באזור מפשעות קו ביקיני.</t>
+        </is>
+      </c>
       <c r="F77" s="3" t="inlineStr"/>
       <c r="G77" s="3" t="inlineStr"/>
       <c r="H77" s="3" t="inlineStr"/>
@@ -5843,7 +6069,11 @@
           <t>מפשעות מלא</t>
         </is>
       </c>
-      <c r="E78" s="3" t="inlineStr"/>
+      <c r="E78" s="3" t="inlineStr">
+        <is>
+          <t>טיפול להסרת שיער באזור מפשעות מלא.</t>
+        </is>
+      </c>
       <c r="F78" s="3" t="inlineStr"/>
       <c r="G78" s="3" t="inlineStr"/>
       <c r="H78" s="3" t="inlineStr"/>
@@ -5881,7 +6111,11 @@
           <t>פס טוסיק ברזילאי</t>
         </is>
       </c>
-      <c r="E79" s="3" t="inlineStr"/>
+      <c r="E79" s="3" t="inlineStr">
+        <is>
+          <t>טיפול להסרת שיער באזור פס טוסיק ברזילאי.</t>
+        </is>
+      </c>
       <c r="F79" s="3" t="inlineStr"/>
       <c r="G79" s="3" t="inlineStr"/>
       <c r="H79" s="3" t="inlineStr"/>
@@ -5919,7 +6153,11 @@
           <t>פס בטן</t>
         </is>
       </c>
-      <c r="E80" s="3" t="inlineStr"/>
+      <c r="E80" s="3" t="inlineStr">
+        <is>
+          <t>טיפול להסרת שיער באזור פס בטן.</t>
+        </is>
+      </c>
       <c r="F80" s="3" t="inlineStr"/>
       <c r="G80" s="3" t="inlineStr"/>
       <c r="H80" s="3" t="inlineStr"/>
@@ -5957,7 +6195,11 @@
           <t>בטן</t>
         </is>
       </c>
-      <c r="E81" s="3" t="inlineStr"/>
+      <c r="E81" s="3" t="inlineStr">
+        <is>
+          <t>טיפול להסרת שיער באזור בטן.</t>
+        </is>
+      </c>
       <c r="F81" s="3" t="inlineStr"/>
       <c r="G81" s="3" t="inlineStr"/>
       <c r="H81" s="3" t="inlineStr"/>
@@ -5995,7 +6237,11 @@
           <t>גב שלם</t>
         </is>
       </c>
-      <c r="E82" s="3" t="inlineStr"/>
+      <c r="E82" s="3" t="inlineStr">
+        <is>
+          <t>טיפול להסרת שיער באזור גב שלם.</t>
+        </is>
+      </c>
       <c r="F82" s="3" t="inlineStr"/>
       <c r="G82" s="3" t="inlineStr"/>
       <c r="H82" s="3" t="inlineStr"/>
@@ -6033,7 +6279,11 @@
           <t>עורף</t>
         </is>
       </c>
-      <c r="E83" s="3" t="inlineStr"/>
+      <c r="E83" s="3" t="inlineStr">
+        <is>
+          <t>טיפול להסרת שיער באזור עורף.</t>
+        </is>
+      </c>
       <c r="F83" s="3" t="inlineStr"/>
       <c r="G83" s="3" t="inlineStr"/>
       <c r="H83" s="3" t="inlineStr"/>
@@ -6071,7 +6321,11 @@
           <t>עורף + כתפיים</t>
         </is>
       </c>
-      <c r="E84" s="3" t="inlineStr"/>
+      <c r="E84" s="3" t="inlineStr">
+        <is>
+          <t>טיפול להסרת שיער באזור עורף + כתפיים.</t>
+        </is>
+      </c>
       <c r="F84" s="3" t="inlineStr"/>
       <c r="G84" s="3" t="inlineStr"/>
       <c r="H84" s="3" t="inlineStr"/>
@@ -6109,7 +6363,11 @@
           <t>גב תחתון</t>
         </is>
       </c>
-      <c r="E85" s="3" t="inlineStr"/>
+      <c r="E85" s="3" t="inlineStr">
+        <is>
+          <t>טיפול להסרת שיער באזור גב תחתון.</t>
+        </is>
+      </c>
       <c r="F85" s="3" t="inlineStr"/>
       <c r="G85" s="3" t="inlineStr"/>
       <c r="H85" s="3" t="inlineStr"/>
@@ -6147,7 +6405,11 @@
           <t>חזה</t>
         </is>
       </c>
-      <c r="E86" s="3" t="inlineStr"/>
+      <c r="E86" s="3" t="inlineStr">
+        <is>
+          <t>טיפול להסרת שיער באזור חזה.</t>
+        </is>
+      </c>
       <c r="F86" s="3" t="inlineStr"/>
       <c r="G86" s="3" t="inlineStr"/>
       <c r="H86" s="3" t="inlineStr"/>
@@ -6185,7 +6447,11 @@
           <t>סביב הפטמות</t>
         </is>
       </c>
-      <c r="E87" s="3" t="inlineStr"/>
+      <c r="E87" s="3" t="inlineStr">
+        <is>
+          <t>טיפול להסרת שיער באזור סביב הפטמות.</t>
+        </is>
+      </c>
       <c r="F87" s="3" t="inlineStr"/>
       <c r="G87" s="3" t="inlineStr"/>
       <c r="H87" s="3" t="inlineStr"/>
@@ -6223,7 +6489,11 @@
           <t>טוסיק פלחים</t>
         </is>
       </c>
-      <c r="E88" s="3" t="inlineStr"/>
+      <c r="E88" s="3" t="inlineStr">
+        <is>
+          <t>טיפול להסרת שיער באזור טוסיק פלחים.</t>
+        </is>
+      </c>
       <c r="F88" s="3" t="inlineStr"/>
       <c r="G88" s="3" t="inlineStr"/>
       <c r="H88" s="3" t="inlineStr"/>
@@ -6261,7 +6531,11 @@
           <t>גוף מלא</t>
         </is>
       </c>
-      <c r="E89" s="3" t="inlineStr"/>
+      <c r="E89" s="3" t="inlineStr">
+        <is>
+          <t>טיפול להסרת שיער באזור גוף מלא.</t>
+        </is>
+      </c>
       <c r="F89" s="3" t="inlineStr"/>
       <c r="G89" s="3" t="inlineStr"/>
       <c r="H89" s="3" t="inlineStr"/>
@@ -6299,7 +6573,11 @@
           <t>שפם</t>
         </is>
       </c>
-      <c r="E90" s="3" t="inlineStr"/>
+      <c r="E90" s="3" t="inlineStr">
+        <is>
+          <t>טיפול להסרת שיער באזור שפם.</t>
+        </is>
+      </c>
       <c r="F90" s="3" t="inlineStr"/>
       <c r="G90" s="3" t="inlineStr"/>
       <c r="H90" s="3" t="inlineStr"/>
@@ -6337,7 +6615,11 @@
           <t>בין הגבות</t>
         </is>
       </c>
-      <c r="E91" s="3" t="inlineStr"/>
+      <c r="E91" s="3" t="inlineStr">
+        <is>
+          <t>טיפול להסרת שיער באזור בין הגבות.</t>
+        </is>
+      </c>
       <c r="F91" s="3" t="inlineStr"/>
       <c r="G91" s="3" t="inlineStr"/>
       <c r="H91" s="3" t="inlineStr"/>
@@ -6375,7 +6657,11 @@
           <t>אוזניים</t>
         </is>
       </c>
-      <c r="E92" s="3" t="inlineStr"/>
+      <c r="E92" s="3" t="inlineStr">
+        <is>
+          <t>טיפול להסרת שיער באזור אוזניים.</t>
+        </is>
+      </c>
       <c r="F92" s="3" t="inlineStr"/>
       <c r="G92" s="3" t="inlineStr"/>
       <c r="H92" s="3" t="inlineStr"/>
@@ -6413,7 +6699,11 @@
           <t>פנים</t>
         </is>
       </c>
-      <c r="E93" s="3" t="inlineStr"/>
+      <c r="E93" s="3" t="inlineStr">
+        <is>
+          <t>טיפול להסרת שיער באזור פנים.</t>
+        </is>
+      </c>
       <c r="F93" s="3" t="inlineStr"/>
       <c r="G93" s="3" t="inlineStr"/>
       <c r="H93" s="3" t="inlineStr"/>
@@ -6447,7 +6737,11 @@
           <t>איפור בוקר</t>
         </is>
       </c>
-      <c r="E94" s="3" t="inlineStr"/>
+      <c r="E94" s="3" t="inlineStr">
+        <is>
+          <t>איפור טבעי ורענן ליום-יום.</t>
+        </is>
+      </c>
       <c r="F94" s="3" t="inlineStr"/>
       <c r="G94" s="3" t="inlineStr"/>
       <c r="H94" s="3" t="inlineStr"/>
@@ -6481,7 +6775,11 @@
           <t>איפור אירועים</t>
         </is>
       </c>
-      <c r="E95" s="3" t="inlineStr"/>
+      <c r="E95" s="3" t="inlineStr">
+        <is>
+          <t>איפור מוקפד ועמיד במיוחד לאירועים.</t>
+        </is>
+      </c>
       <c r="F95" s="3" t="inlineStr"/>
       <c r="G95" s="3" t="inlineStr"/>
       <c r="H95" s="3" t="inlineStr"/>
@@ -6515,7 +6813,11 @@
           <t>איפור + עיצוב שיער לאירוע</t>
         </is>
       </c>
-      <c r="E96" s="3" t="inlineStr"/>
+      <c r="E96" s="3" t="inlineStr">
+        <is>
+          <t>חבילת איפור לאירוע בשילוב עיצוב שיער.</t>
+        </is>
+      </c>
       <c r="F96" s="3" t="inlineStr"/>
       <c r="G96" s="3" t="inlineStr"/>
       <c r="H96" s="3" t="inlineStr"/>
@@ -7367,7 +7669,11 @@
           <t>נקודת חן</t>
         </is>
       </c>
-      <c r="E107" s="3" t="inlineStr"/>
+      <c r="E107" s="3" t="inlineStr">
+        <is>
+          <t>טיפול איפור קבוע להוספת נקודת חן.</t>
+        </is>
+      </c>
       <c r="F107" s="3" t="inlineStr"/>
       <c r="G107" s="3" t="inlineStr"/>
       <c r="H107" s="3" t="inlineStr"/>
@@ -7405,7 +7711,11 @@
           <t>איילינר תחתון</t>
         </is>
       </c>
-      <c r="E108" s="3" t="inlineStr"/>
+      <c r="E108" s="3" t="inlineStr">
+        <is>
+          <t>תיחום והדגשה של קו העיניים.</t>
+        </is>
+      </c>
       <c r="F108" s="3" t="inlineStr"/>
       <c r="G108" s="3" t="inlineStr"/>
       <c r="H108" s="3" t="inlineStr"/>
@@ -7443,7 +7753,11 @@
           <t>איילינר מעושן עד 3 צבעים</t>
         </is>
       </c>
-      <c r="E109" s="3" t="inlineStr"/>
+      <c r="E109" s="3" t="inlineStr">
+        <is>
+          <t>תיחום והדגשה של קו העיניים.</t>
+        </is>
+      </c>
       <c r="F109" s="3" t="inlineStr"/>
       <c r="G109" s="3" t="inlineStr"/>
       <c r="H109" s="3" t="inlineStr"/>
@@ -7481,7 +7795,11 @@
           <t>החלקת/הרמת גבות - עיצוב+צבע+הרמה</t>
         </is>
       </c>
-      <c r="E110" s="3" t="inlineStr"/>
+      <c r="E110" s="3" t="inlineStr">
+        <is>
+          <t>טיפול לעיצוב, סידור וטיפוח הגבות.</t>
+        </is>
+      </c>
       <c r="F110" s="3" t="inlineStr"/>
       <c r="G110" s="3" t="inlineStr"/>
       <c r="H110" s="3" t="inlineStr"/>
@@ -7523,7 +7841,11 @@
           <t>סידור ועיצוב גבות</t>
         </is>
       </c>
-      <c r="E111" s="3" t="inlineStr"/>
+      <c r="E111" s="3" t="inlineStr">
+        <is>
+          <t>טיפול לעיצוב, סידור וטיפוח הגבות.</t>
+        </is>
+      </c>
       <c r="F111" s="3" t="inlineStr"/>
       <c r="G111" s="3" t="inlineStr"/>
       <c r="H111" s="3" t="inlineStr"/>
@@ -7561,7 +7883,11 @@
           <t>גבות + שפם</t>
         </is>
       </c>
-      <c r="E112" s="3" t="inlineStr"/>
+      <c r="E112" s="3" t="inlineStr">
+        <is>
+          <t>טיפול לעיצוב, סידור וטיפוח הגבות.</t>
+        </is>
+      </c>
       <c r="F112" s="3" t="inlineStr"/>
       <c r="G112" s="3" t="inlineStr"/>
       <c r="H112" s="3" t="inlineStr"/>
@@ -7599,7 +7925,11 @@
           <t>צבע ריסים</t>
         </is>
       </c>
-      <c r="E113" s="3" t="inlineStr"/>
+      <c r="E113" s="3" t="inlineStr">
+        <is>
+          <t>טיפול לעיצוב, צביעה או הדגשה של הריסים.</t>
+        </is>
+      </c>
       <c r="F113" s="3" t="inlineStr"/>
       <c r="G113" s="3" t="inlineStr"/>
       <c r="H113" s="3" t="inlineStr"/>
@@ -7637,7 +7967,11 @@
           <t>צבע ריסים + גבות</t>
         </is>
       </c>
-      <c r="E114" s="3" t="inlineStr"/>
+      <c r="E114" s="3" t="inlineStr">
+        <is>
+          <t>טיפול לעיצוב, צביעה או הדגשה של הריסים.</t>
+        </is>
+      </c>
       <c r="F114" s="3" t="inlineStr"/>
       <c r="G114" s="3" t="inlineStr"/>
       <c r="H114" s="3" t="inlineStr"/>
@@ -7675,7 +8009,11 @@
           <t>עיצוב וסידור גבות + צבע</t>
         </is>
       </c>
-      <c r="E115" s="3" t="inlineStr"/>
+      <c r="E115" s="3" t="inlineStr">
+        <is>
+          <t>טיפול לעיצוב, סידור וטיפוח הגבות.</t>
+        </is>
+      </c>
       <c r="F115" s="3" t="inlineStr"/>
       <c r="G115" s="3" t="inlineStr"/>
       <c r="H115" s="3" t="inlineStr"/>
@@ -7713,7 +8051,11 @@
           <t>שפם</t>
         </is>
       </c>
-      <c r="E116" s="3" t="inlineStr"/>
+      <c r="E116" s="3" t="inlineStr">
+        <is>
+          <t>טיפול לעיצוב או להסרת שיער השפם.</t>
+        </is>
+      </c>
       <c r="F116" s="3" t="inlineStr"/>
       <c r="G116" s="3" t="inlineStr"/>
       <c r="H116" s="3" t="inlineStr"/>
@@ -7751,7 +8093,11 @@
           <t>הרמת ריסים</t>
         </is>
       </c>
-      <c r="E117" s="3" t="inlineStr"/>
+      <c r="E117" s="3" t="inlineStr">
+        <is>
+          <t>טיפול לעיצוב, צביעה או הדגשה של הריסים.</t>
+        </is>
+      </c>
       <c r="F117" s="3" t="inlineStr"/>
       <c r="G117" s="3" t="inlineStr"/>
       <c r="H117" s="3" t="inlineStr"/>
@@ -7865,7 +8211,11 @@
           <t>Botox (אזור בודד)</t>
         </is>
       </c>
-      <c r="E120" s="3" t="inlineStr"/>
+      <c r="E120" s="3" t="inlineStr">
+        <is>
+          <t>טיפול בתחום האסתטיקה, מותאם אישית. הצוות המקצועי שלנו ישמח לייעץ ולהתאים את הטיפול עבורך.</t>
+        </is>
+      </c>
       <c r="F120" s="3" t="inlineStr"/>
       <c r="G120" s="3" t="inlineStr"/>
       <c r="H120" s="3" t="inlineStr"/>
@@ -7907,7 +8257,11 @@
           <t>Botox (3 אזורים)</t>
         </is>
       </c>
-      <c r="E121" s="3" t="inlineStr"/>
+      <c r="E121" s="3" t="inlineStr">
+        <is>
+          <t>טיפול בתחום האסתטיקה, מותאם אישית. הצוות המקצועי שלנו ישמח לייעץ ולהתאים את הטיפול עבורך.</t>
+        </is>
+      </c>
       <c r="F121" s="3" t="inlineStr"/>
       <c r="G121" s="3" t="inlineStr"/>
       <c r="H121" s="3" t="inlineStr"/>
@@ -7995,7 +8349,11 @@
           <t>Gummy smile Botox</t>
         </is>
       </c>
-      <c r="E123" s="3" t="inlineStr"/>
+      <c r="E123" s="3" t="inlineStr">
+        <is>
+          <t>טיפול בתחום האסתטיקה, מותאם אישית. הצוות המקצועי שלנו ישמח לייעץ ולהתאים את הטיפול עבורך.</t>
+        </is>
+      </c>
       <c r="F123" s="3" t="inlineStr"/>
       <c r="G123" s="3" t="inlineStr"/>
       <c r="H123" s="3" t="inlineStr"/>
@@ -8037,7 +8395,11 @@
           <t>Lip filler (Stylage/Restylane)</t>
         </is>
       </c>
-      <c r="E124" s="3" t="inlineStr"/>
+      <c r="E124" s="3" t="inlineStr">
+        <is>
+          <t>טיפול בתחום האסתטיקה, מותאם אישית. הצוות המקצועי שלנו ישמח לייעץ ולהתאים את הטיפול עבורך.</t>
+        </is>
+      </c>
       <c r="F124" s="3" t="inlineStr"/>
       <c r="G124" s="3" t="inlineStr"/>
       <c r="H124" s="3" t="inlineStr"/>
@@ -8079,7 +8441,11 @@
           <t>Filler Restylane (Stylage/Restylane)</t>
         </is>
       </c>
-      <c r="E125" s="3" t="inlineStr"/>
+      <c r="E125" s="3" t="inlineStr">
+        <is>
+          <t>טיפול בתחום האסתטיקה, מותאם אישית. הצוות המקצועי שלנו ישמח לייעץ ולהתאים את הטיפול עבורך.</t>
+        </is>
+      </c>
       <c r="F125" s="3" t="inlineStr"/>
       <c r="G125" s="3" t="inlineStr"/>
       <c r="H125" s="3" t="inlineStr"/>
@@ -8121,7 +8487,11 @@
           <t>Radiesse</t>
         </is>
       </c>
-      <c r="E126" s="3" t="inlineStr"/>
+      <c r="E126" s="3" t="inlineStr">
+        <is>
+          <t>טיפול בתחום האסתטיקה, מותאם אישית. הצוות המקצועי שלנו ישמח לייעץ ולהתאים את הטיפול עבורך.</t>
+        </is>
+      </c>
       <c r="F126" s="3" t="inlineStr"/>
       <c r="G126" s="3" t="inlineStr"/>
       <c r="H126" s="3" t="inlineStr"/>
@@ -8293,7 +8663,11 @@
           <t>Cellboster (סקין בוסטר)</t>
         </is>
       </c>
-      <c r="E130" s="3" t="inlineStr"/>
+      <c r="E130" s="3" t="inlineStr">
+        <is>
+          <t>טיפול בתחום האסתטיקה, מותאם אישית. הצוות המקצועי שלנו ישמח לייעץ ולהתאים את הטיפול עבורך.</t>
+        </is>
+      </c>
       <c r="F130" s="3" t="inlineStr"/>
       <c r="G130" s="3" t="inlineStr"/>
       <c r="H130" s="3" t="inlineStr"/>
@@ -8331,7 +8705,11 @@
           <t>Karisma (סקין בוסטר)</t>
         </is>
       </c>
-      <c r="E131" s="3" t="inlineStr"/>
+      <c r="E131" s="3" t="inlineStr">
+        <is>
+          <t>טיפול בתחום האסתטיקה, מותאם אישית. הצוות המקצועי שלנו ישמח לייעץ ולהתאים את הטיפול עבורך.</t>
+        </is>
+      </c>
       <c r="F131" s="3" t="inlineStr"/>
       <c r="G131" s="3" t="inlineStr"/>
       <c r="H131" s="3" t="inlineStr"/>
@@ -8369,7 +8747,11 @@
           <t>פולינוקליאוטידים - זרעי סלמון</t>
         </is>
       </c>
-      <c r="E132" s="3" t="inlineStr"/>
+      <c r="E132" s="3" t="inlineStr">
+        <is>
+          <t>טיפול בתחום האסתטיקה, מותאם אישית. הצוות המקצועי שלנו ישמח לייעץ ולהתאים את הטיפול עבורך.</t>
+        </is>
+      </c>
       <c r="F132" s="3" t="inlineStr"/>
       <c r="G132" s="3" t="inlineStr"/>
       <c r="H132" s="3" t="inlineStr"/>
@@ -8411,7 +8793,11 @@
           <t>Antiage Skinpen</t>
         </is>
       </c>
-      <c r="E133" s="3" t="inlineStr"/>
+      <c r="E133" s="3" t="inlineStr">
+        <is>
+          <t>טיפול בתחום האסתטיקה, מותאם אישית. הצוות המקצועי שלנו ישמח לייעץ ולהתאים את הטיפול עבורך.</t>
+        </is>
+      </c>
       <c r="F133" s="3" t="inlineStr"/>
       <c r="G133" s="3" t="inlineStr"/>
       <c r="H133" s="3" t="inlineStr"/>
@@ -8495,7 +8881,11 @@
           <t>Dermapen + Biorepeel</t>
         </is>
       </c>
-      <c r="E135" s="3" t="inlineStr"/>
+      <c r="E135" s="3" t="inlineStr">
+        <is>
+          <t>טיפול בתחום האסתטיקה, מותאם אישית. הצוות המקצועי שלנו ישמח לייעץ ולהתאים את הטיפול עבורך.</t>
+        </is>
+      </c>
       <c r="F135" s="3" t="inlineStr"/>
       <c r="G135" s="3" t="inlineStr"/>
       <c r="H135" s="3" t="inlineStr"/>
@@ -8537,7 +8927,11 @@
           <t>חבילת שיפור והצערה משולבת (Sculptra + זרעי סלמון)</t>
         </is>
       </c>
-      <c r="E136" s="3" t="inlineStr"/>
+      <c r="E136" s="3" t="inlineStr">
+        <is>
+          <t>טיפול בתחום האסתטיקה, מותאם אישית. הצוות המקצועי שלנו ישמח לייעץ ולהתאים את הטיפול עבורך.</t>
+        </is>
+      </c>
       <c r="F136" s="3" t="inlineStr"/>
       <c r="G136" s="3" t="inlineStr"/>
       <c r="H136" s="3" t="inlineStr"/>

</xml_diff>